<commit_message>
data: oportunidades Visión Circular 2026-09-11
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI266"/>
+  <dimension ref="A1:AI270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41274,7 +41274,7 @@
       </c>
       <c r="AD231" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AE231" t="inlineStr">
@@ -41284,7 +41284,7 @@
       </c>
       <c r="AF231" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AG231" t="inlineStr">
@@ -41299,7 +41299,7 @@
       </c>
       <c r="AI231" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -45088,7 +45088,7 @@
       </c>
       <c r="N253" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Abierta permanentemente (según anuncio de lanzamiento)</t>
         </is>
       </c>
       <c r="O253" t="inlineStr">
@@ -45178,7 +45178,7 @@
       </c>
       <c r="AF253" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AG253" t="inlineStr">
@@ -45193,7 +45193,7 @@
       </c>
       <c r="AI253" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -47495,6 +47495,714 @@
       <c r="AI266" t="inlineStr">
         <is>
           <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>VC-0266</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Circulate Capital – Funding for Recycling Supply Chains</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Circulate Capital</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Global (incluye Colombia y América Latina)</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Reciclaje</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Cadena de suministro de reciclaje; Upcycling; Digitalización</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Cofinanciación</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N267" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q267" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R267" t="inlineStr">
+        <is>
+          <t>https://www.circulatecapital.com/apply-for-funding</t>
+        </is>
+      </c>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr">
+        <is>
+          <t>Circulate Capital ofrece financiamiento (equity o deuda) a empresas que desarrollen soluciones de recolección, clasificación, upcycling y digitalización de la cadena de reciclaje en América Latina, con foco en escalabilidad e impacto ambiental.</t>
+        </is>
+      </c>
+      <c r="U267" t="inlineStr">
+        <is>
+          <t>Apoya directamente la mejora de la recolección y reciclabilidad de envases, la inclusión de recicladores y la digitalización de la cadena, pilares de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V267" t="inlineStr">
+        <is>
+          <t>Plataformas de trazabilidad y datos para envases; Tecnologías de clasificación y upcycling de plásticos flexibles; Soluciones de logística inversa; Modelos de negocio inclusivos para recicladores informales.</t>
+        </is>
+      </c>
+      <c r="W267" t="inlineStr">
+        <is>
+          <t>Ser empresa operante en la cadena de reciclaje; Modelo de negocio escalable; Evidencia de impacto ambiental medible; Capacidad de reportar métricas financieras.</t>
+        </is>
+      </c>
+      <c r="X267" t="inlineStr">
+        <is>
+          <t>Pitch deck; Plan de negocio; Proyecciones financieras; Métricas de impacto; Información legal de la entidad.</t>
+        </is>
+      </c>
+      <c r="Y267" t="inlineStr">
+        <is>
+          <t>ANDI, gremios de envases y empaques, universidades de ingeniería y diseño, asociaciones de recicladores, agencias de desarrollo regional.</t>
+        </is>
+      </c>
+      <c r="Z267" t="inlineStr">
+        <is>
+          <t>Requisitos de retorno financiero; Necesidad de co‑inversión; Posible enfoque en empresas con modelo de negocio comercial más que en ONGs.</t>
+        </is>
+      </c>
+      <c r="AA267" t="inlineStr">
+        <is>
+          <t>Revisar criterios de elegibilidad y preparar dossier de inversión alineado con los objetivos de Circulate Capital.</t>
+        </is>
+      </c>
+      <c r="AB267" t="inlineStr">
+        <is>
+          <t>Completar el formulario de contacto en la página oficial y solicitar guía de aplicación específica para Colombia.</t>
+        </is>
+      </c>
+      <c r="AC267" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas estratégicas / Gestión de proyectos de innovación</t>
+        </is>
+      </c>
+      <c r="AD267" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE267" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF267" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG267" t="inlineStr">
+        <is>
+          <t>La página no indica fecha límite ni monto máximo; se asume proceso continuo y abierto a propuestas de cualquier país elegible.</t>
+        </is>
+      </c>
+      <c r="AH267" t="inlineStr">
+        <is>
+          <t>d5955d48b3ca1093</t>
+        </is>
+      </c>
+      <c r="AI267" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>VC-0267</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Horizon Europe 2025 – Grant for Eco‑Friendly Packaging (Circular design of fiber‑based packaging with enhanced functionalities)</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>European Commission – Horizon Europe Programme</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Estados miembros de la UE, países asociados al programa y terceros países mediante consorcio con entidad elegible</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Eco‑diseño y materiales de envases sostenibles (fibra, biodegradable)</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Investigación aplicada; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N268" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P268" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q268" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R268" t="inlineStr">
+        <is>
+          <t>https://getgrant.eu/grants-and-funding/grant-for-eco-friendly-packaging-horizon-europe-2025-call-for-innovative-materials</t>
+        </is>
+      </c>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T268" t="inlineStr">
+        <is>
+          <t>Financia proyectos de I+D+i que desarrollen diseños circulares para envases de fibra con funcionalidades mejoradas, con el objetivo de reducir la dependencia de plásticos y mejorar la reciclabilidad. El apoyo cubre actividades de investigación, prototipado y pruebas piloto.</t>
+        </is>
+      </c>
+      <c r="U268" t="inlineStr">
+        <is>
+          <t>Apoya directamente la línea de trabajo de Visión Circular en ecodiseño, reciclabilidad y sustitución de plásticos en envases y empaques.</t>
+        </is>
+      </c>
+      <c r="V268" t="inlineStr">
+        <is>
+          <t>Desarrollo de envases de fibra con alta resistencia; pruebas de reciclabilidad; estudios de ciclo de vida; integración de recicladores en la cadena de valor.</t>
+        </is>
+      </c>
+      <c r="W268" t="inlineStr">
+        <is>
+          <t>Consorcio con al menos una entidad elegible de la UE; proyecto de 24‑36 meses; presupuesto total ≤ 5 M EUR; alineación con los objetivos de la llamada.</t>
+        </is>
+      </c>
+      <c r="X268" t="inlineStr">
+        <is>
+          <t>Formulario de propuesta, plan de trabajo, presupuesto detallado, cartas de compromiso de socios, evidencia de capacidad técnica.</t>
+        </is>
+      </c>
+      <c r="Y268" t="inlineStr">
+        <is>
+          <t>Universidades e I+D colombianas, asociaciones de recicladores, cámaras de envases y empaques, centros de innovación tecnológica.</t>
+        </is>
+      </c>
+      <c r="Z268" t="inlineStr">
+        <is>
+          <t>Necesidad de socio europeo para elegibilidad; alta competencia; cumplimiento de requisitos de reporte financiero UE.</t>
+        </is>
+      </c>
+      <c r="AA268" t="inlineStr">
+        <is>
+          <t>Identificar y contactar potenciales socios europeos (universidades, empresas) para formar consorcio antes de la fecha límite.</t>
+        </is>
+      </c>
+      <c r="AB268" t="inlineStr">
+        <is>
+          <t>Revisar la guía completa de la convocatoria en la página oficial y elaborar una lista preliminar de socios estratégicos en Europa.</t>
+        </is>
+      </c>
+      <c r="AC268" t="inlineStr">
+        <is>
+          <t>Coordinación de Alianzas Estratégicas y Proyectos de Innovación</t>
+        </is>
+      </c>
+      <c r="AD268" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE268" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF268" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG268" t="inlineStr">
+        <is>
+          <t>La convocatoria está publicada, pero la fecha exacta de cierre no aparece en la fuente consultada; se asume que sigue abierta o se abrirá pronto. | Fuente fuera del listado oficial conocido (getgrant.eu): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH268" t="inlineStr">
+        <is>
+          <t>277fd768a8d72f12</t>
+        </is>
+      </c>
+      <c r="AI268" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>VC-0268</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>EU Funding – Call for proposals on circularity of multilayer flexible plastic food‑contact packaging</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>European Commission – Horizon Europe / EU Funding Portal</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Estados miembros de la UE, países asociados y terceros países mediante consorcio con entidad elegible</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Plásticos flexibles, reciclabilidad de envases alimentarios</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N269" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q269" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R269" t="inlineStr">
+        <is>
+          <t>https://eufundingportal.eu/circular-economy</t>
+        </is>
+      </c>
+      <c r="S269" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T269" t="inlineStr">
+        <is>
+          <t>Financia proyectos que desarrollen soluciones innovadoras para mejorar la circularidad de empaques multilayer flexibles en contacto con alimentos, incluyendo nuevas materias primas, procesos de reciclaje y modelos de negocio circulares.</t>
+        </is>
+      </c>
+      <c r="U269" t="inlineStr">
+        <is>
+          <t>Se alinea con los objetivos de Visión Circular de cerrar el ciclo de plásticos flexibles y promover la inclusión de recicladores en la cadena de valor.</t>
+        </is>
+      </c>
+      <c r="V269" t="inlineStr">
+        <is>
+          <t>Desarrollo de materiales alternativos; tecnologías de reciclaje de multilayer; plataformas de trazabilidad; modelos de negocio de retorno y reutilización.</t>
+        </is>
+      </c>
+      <c r="W269" t="inlineStr">
+        <is>
+          <t>Consorcio con al menos una entidad elegible de la UE; proyecto de 2‑3 años; presupuesto total ≤ 4 M EUR; cumplimiento de normas de seguridad alimentaria.</t>
+        </is>
+      </c>
+      <c r="X269" t="inlineStr">
+        <is>
+          <t>Propuesta técnica, plan de gestión, presupuesto, cartas de intención de socios, certificaciones de cumplimiento de normas alimentarias.</t>
+        </is>
+      </c>
+      <c r="Y269" t="inlineStr">
+        <is>
+          <t>Empresas colombianas de envases flexibles, centros de investigación de alimentos, asociaciones de recicladores, universidades con líneas de investigación en polímeros.</t>
+        </is>
+      </c>
+      <c r="Z269" t="inlineStr">
+        <is>
+          <t>Requisitos estrictos de seguridad alimentaria; necesidad de socios europeos; posible limitación de fondos para terceros países.</t>
+        </is>
+      </c>
+      <c r="AA269" t="inlineStr">
+        <is>
+          <t>Mapear actores locales en la cadena de empaques flexibles y buscar alianzas con universidades o empresas europeas que ya participen en proyectos Horizon.</t>
+        </is>
+      </c>
+      <c r="AB269" t="inlineStr">
+        <is>
+          <t>Acceder al portal EU Funding, descargar el documento de la convocatoria y revisar los criterios de elegibilidad para terceros países.</t>
+        </is>
+      </c>
+      <c r="AC269" t="inlineStr">
+        <is>
+          <t>Unidad de Innovación y Desarrollo de Productos Sustentables</t>
+        </is>
+      </c>
+      <c r="AD269" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE269" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF269" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG269" t="inlineStr">
+        <is>
+          <t>La convocatoria aparece en el portal oficial, pero la fecha de cierre no está visible; se requiere confirmar vigencia y requisitos de participación de Colombia. | Fuente fuera del listado oficial conocido (eufundingportal.eu): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH269" t="inlineStr">
+        <is>
+          <t>1ee59e50c04a96c7</t>
+        </is>
+      </c>
+      <c r="AI269" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>VC-0269</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Convocatoria LIFE 2026 – Economía circular y contaminación cero</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Comisión Europea – Programa LIFE</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Estados miembros de la UE y países asociados (verificar si Colombia puede participar como socio)</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Economía circular y contaminación cero</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>Sí / Descripción</t>
+        </is>
+      </c>
+      <c r="N270" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q270" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R270" t="inlineStr">
+        <is>
+          <t>https://www.zabala.es/noticias/convocatoria-life</t>
+        </is>
+      </c>
+      <c r="S270" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T270" t="inlineStr">
+        <is>
+          <t>Financia proyectos de acción estándar (SAP) que demuestren enfoques innovadores en economía circular y contaminación cero, con miras a replicar a mayor escala. La convocatoria está dirigida a entidades elegibles dentro del marco del programa LIFE 2026.</t>
+        </is>
+      </c>
+      <c r="U270" t="inlineStr">
+        <is>
+          <t>Apoya directamente la agenda de economía circular, reciclaje y reducción de residuos, áreas centrales de Visión Circular de la ANDI.</t>
+        </is>
+      </c>
+      <c r="V270" t="inlineStr">
+        <is>
+          <t>Desarrollo de modelos de negocio circulares; Pilotos de reciclaje de envases y empaques; Innovación en ecodiseño de plásticos flexibles; Inclusión de recicladores en cadenas de valor.</t>
+        </is>
+      </c>
+      <c r="W270" t="inlineStr">
+        <is>
+          <t>Ser entidad elegible según criterios LIFE (empresa, ONG, universidad, autoridad pública); presentar proyecto alineado con los objetivos de economía circular; cofinanciación requerida.</t>
+        </is>
+      </c>
+      <c r="X270" t="inlineStr">
+        <is>
+          <t>Formulario de solicitud LIFE; plan de proyecto; presupuesto detallado; evidencia de capacidad técnica; cartas de apoyo de socios.</t>
+        </is>
+      </c>
+      <c r="Y270" t="inlineStr">
+        <is>
+          <t>Universidades e institutos de investigación; gremios de la industria de envases; asociaciones de recicladores; agencias de cooperación internacional.</t>
+        </is>
+      </c>
+      <c r="Z270" t="inlineStr">
+        <is>
+          <t>Elegibilidad limitada a países asociados; proceso de revisión competitivo y exigente; necesidad de cofinanciación.</t>
+        </is>
+      </c>
+      <c r="AA270" t="inlineStr">
+        <is>
+          <t>Verificar la posibilidad de presentar la propuesta como socio de una entidad europea elegible o a través de un consorcio internacional.</t>
+        </is>
+      </c>
+      <c r="AB270" t="inlineStr">
+        <is>
+          <t>Consultar la guía oficial LIFE 2026 y contactar la oficina de la UE en Bogotá para confirmar vías de participación.</t>
+        </is>
+      </c>
+      <c r="AC270" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos internacionales</t>
+        </is>
+      </c>
+      <c r="AD270" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE270" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF270" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG270" t="inlineStr">
+        <is>
+          <t>La convocatoria es real y vigente, pero la elegibilidad de Colombia no está clara; se requiere confirmación de posibilidad de participación como socio o mediante consorcio. | Fuente fuera del listado oficial conocido (zabala.es): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH270" t="inlineStr">
+        <is>
+          <t>e8e7f4bd08d9584d</t>
+        </is>
+      </c>
+      <c r="AI270" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-09-18
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI270"/>
+  <dimension ref="A1:AI275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46938,7 +46938,7 @@
       </c>
       <c r="AD263" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AE263" t="inlineStr">
@@ -46948,7 +46948,7 @@
       </c>
       <c r="AF263" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AG263" t="inlineStr">
@@ -46963,7 +46963,7 @@
       </c>
       <c r="AI263" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -48203,6 +48203,891 @@
       <c r="AI270" t="inlineStr">
         <is>
           <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>VC-0270</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Convocatoria Portafolio de Oferta de Cooperación Internacional 2024-2025</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Agencia Presidencial de Cooperación Internacional (APC-Colombia)</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Gobierno</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Cooperación técnica</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>https://www.apccolombia.gov.co/modalidades-de-cooperacion/convocatorias/convocatoria-portafolio-de-oferta/convocatoria-portafolio</t>
+        </is>
+      </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T271" t="inlineStr">
+        <is>
+          <t>La convocatoria busca fortalecer capacidades en Colombia a través de intercambios de conocimiento y tecnología, con enfoque en los Objetivos de Desarrollo Sostenible. Los proyectos deben presentar propuestas de cooperación internacional y pueden incluir componentes de economía circular. Los plazos y montos exactos no se han publicado aún.</t>
+        </is>
+      </c>
+      <c r="U271" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular por su enfoque en desarrollo sostenible y potencial de incluir proyectos de economía circular y reciclaje.</t>
+        </is>
+      </c>
+      <c r="V271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="W271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Z271" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AA271" t="inlineStr">
+        <is>
+          <t>Monitorear la página de APC para fechas y requisitos.</t>
+        </is>
+      </c>
+      <c r="AB271" t="inlineStr">
+        <is>
+          <t>Revisar la convocatoria y preparar propuesta.</t>
+        </is>
+      </c>
+      <c r="AC271" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos</t>
+        </is>
+      </c>
+      <c r="AD271" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE271" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF271" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG271" t="inlineStr">
+        <is>
+          <t>La convocatoria está anunciada pero no se han publicado fechas ni montos. Se requiere verificación de vigencia y requisitos.</t>
+        </is>
+      </c>
+      <c r="AH271" t="inlineStr">
+        <is>
+          <t>39015036ab8d6b13</t>
+        </is>
+      </c>
+      <c r="AI271" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>VC-0271</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Premio Ambiental CAR – Colombia Líder</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Corporación Autónoma Regional de Cundinamarca (CAR)</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Gobierno | Agencia regional</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Sostenibilidad ambiental</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Buenas prácticas ambientales, protección ambiental</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R272" t="inlineStr">
+        <is>
+          <t>https://www.colombialider.org/carpremiacion</t>
+        </is>
+      </c>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T272" t="inlineStr">
+        <is>
+          <t>Premio que reconoce proyectos y liderazgos que contribuyen a la protección y sostenibilidad ambiental en Cundinamarca. Se busca destacar buenas prácticas locales con impacto ambiental positivo.</t>
+        </is>
+      </c>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>Relevante por su enfoque en sostenibilidad y protección ambiental, alineado con la economía circular y la gestión de residuos.</t>
+        </is>
+      </c>
+      <c r="V272" t="inlineStr">
+        <is>
+          <t>Implementación de sistemas de reciclaje, diseño de empaques sostenibles, inclusión de recicladores.</t>
+        </is>
+      </c>
+      <c r="W272" t="inlineStr">
+        <is>
+          <t>Proyecto con impacto ambiental positivo en Cundinamarca, demostrable.</t>
+        </is>
+      </c>
+      <c r="X272" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto, documentación de impacto, certificaciones.</t>
+        </is>
+      </c>
+      <c r="Y272" t="inlineStr">
+        <is>
+          <t>Empresas locales, universidades, ONG ambientales.</t>
+        </is>
+      </c>
+      <c r="Z272" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AA272" t="inlineStr">
+        <is>
+          <t>Consultar la página para confirmar vigencia y requisitos.</t>
+        </is>
+      </c>
+      <c r="AB272" t="inlineStr">
+        <is>
+          <t>Revisar la convocatoria y preparar documentación.</t>
+        </is>
+      </c>
+      <c r="AC272" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos</t>
+        </is>
+      </c>
+      <c r="AD272" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE272" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF272" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG272" t="inlineStr">
+        <is>
+          <t>Requiere verificación de vigencia y elegibilidad. | Fuente fuera del listado oficial conocido (colombialider.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH272" t="inlineStr">
+        <is>
+          <t>ad9e65873c63ef62</t>
+        </is>
+      </c>
+      <c r="AI272" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>VC-0272</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Premio Ambiental Gemas</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Fundación Gemas</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Fundación</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Sostenibilidad ambiental</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Protección ambiental</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R273" t="inlineStr">
+        <is>
+          <t>https://premiogemas.co</t>
+        </is>
+      </c>
+      <c r="S273" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T273" t="inlineStr">
+        <is>
+          <t>Premio que reconoce y premia el trabajo de personas, organizaciones e instituciones que lideran acciones para proteger el medio ambiente en Colombia.</t>
+        </is>
+      </c>
+      <c r="U273" t="inlineStr">
+        <is>
+          <t>Alineado con la promoción de prácticas sostenibles y la economía circular.</t>
+        </is>
+      </c>
+      <c r="V273" t="inlineStr">
+        <is>
+          <t>Iniciativas de reciclaje, diseño de empaques sostenibles, inclusión de recicladores.</t>
+        </is>
+      </c>
+      <c r="W273" t="inlineStr">
+        <is>
+          <t>Proyecto con impacto ambiental positivo.</t>
+        </is>
+      </c>
+      <c r="X273" t="inlineStr">
+        <is>
+          <t>Propuesta, documentación de impacto.</t>
+        </is>
+      </c>
+      <c r="Y273" t="inlineStr">
+        <is>
+          <t>Empresas, universidades, ONG.</t>
+        </is>
+      </c>
+      <c r="Z273" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AA273" t="inlineStr">
+        <is>
+          <t>Verificar vigencia y requisitos.</t>
+        </is>
+      </c>
+      <c r="AB273" t="inlineStr">
+        <is>
+          <t>Consultar la convocatoria.</t>
+        </is>
+      </c>
+      <c r="AC273" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos</t>
+        </is>
+      </c>
+      <c r="AD273" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE273" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF273" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG273" t="inlineStr">
+        <is>
+          <t>Requiere verificación de vigencia y elegibilidad. | Fuente fuera del listado oficial conocido (premiogemas.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH273" t="inlineStr">
+        <is>
+          <t>5f935d670396a8dd</t>
+        </is>
+      </c>
+      <c r="AI273" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>VC-0273</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>21.º Premio Andesco a la Sostenibilidad - Pacto Global Red Colombia</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Pacto Global Red Colombia</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>ONG</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Innovación ambiental</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N274" t="inlineStr">
+        <is>
+          <t>2024-02-10</t>
+        </is>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>2024-04-30</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R274" t="inlineStr">
+        <is>
+          <t>https://www.pactoglobal-colombia.org/news/ya-esta-abierta-la-convocatoria-al-21-o-premio-andesco-a-la-sostenibilidad.html</t>
+        </is>
+      </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr">
+        <is>
+          <t>Premio que reconoce las mejores prácticas empresariales en sostenibilidad, con enfoque en innovación ambiental y modelos circulares. Se invita a empresas, organizaciones y emprendedores a presentar proyectos con impacto positivo.</t>
+        </is>
+      </c>
+      <c r="U274" t="inlineStr">
+        <is>
+          <t>Relevante por su enfoque en modelos circulares y sostenibilidad empresarial, alineado con Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V274" t="inlineStr">
+        <is>
+          <t>Desarrollo de modelos de negocio circulares, ecodiseño, inclusión de recicladores, cumplimiento de REP.</t>
+        </is>
+      </c>
+      <c r="W274" t="inlineStr">
+        <is>
+          <t>Ser empresa o entidad con proyecto de sostenibilidad; presentar propuesta de proyecto; cumplir con criterios de innovación y impacto ambiental.</t>
+        </is>
+      </c>
+      <c r="X274" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto, plan de trabajo, presupuesto, datos de impacto, documentación legal.</t>
+        </is>
+      </c>
+      <c r="Y274" t="inlineStr">
+        <is>
+          <t>Gremios empresariales, universidades, centros de investigación, recicladores, entidades de cooperación.</t>
+        </is>
+      </c>
+      <c r="Z274" t="inlineStr">
+        <is>
+          <t>Competencia alta; requisitos de presentación; falta de claridad en criterios de evaluación.</t>
+        </is>
+      </c>
+      <c r="AA274" t="inlineStr">
+        <is>
+          <t>Preparar propuesta de proyecto alineada con criterios de innovación y sostenibilidad; contactar con Pacto Global Red Colombia para aclarar dudas.</t>
+        </is>
+      </c>
+      <c r="AB274" t="inlineStr">
+        <is>
+          <t>Revisar requisitos en la convocatoria y comenzar la preparación de la propuesta.</t>
+        </is>
+      </c>
+      <c r="AC274" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas</t>
+        </is>
+      </c>
+      <c r="AD274" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE274" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF274" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG274" t="inlineStr">
+        <is>
+          <t>La convocatoria está abierta del 10 de febrero al 30 de abril de 2024. Se requiere confirmar los criterios de evaluación y monto del premio. | Fuente fuera del listado oficial conocido (pactoglobal-colombia.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH274" t="inlineStr">
+        <is>
+          <t>217125bc76775c1d</t>
+        </is>
+      </c>
+      <c r="AI274" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>VC-0274</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>IKI Country Call Colombia 2024</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Internationale Klimaschutzinitiative (IKI)</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Innovación climática</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R275" t="inlineStr">
+        <is>
+          <t>https://www.international-climate-initiative.com/en/find-funding/country-call/country-call-colombia-2024</t>
+        </is>
+      </c>
+      <c r="S275" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T275" t="inlineStr">
+        <is>
+          <t>Ideas competition for climate solutions in Colombia, open to Colombian organizations, with potential funding and technical support.</t>
+        </is>
+      </c>
+      <c r="U275" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular porque promueve innovación climática y puede incluir proyectos de economía circular.</t>
+        </is>
+      </c>
+      <c r="V275" t="inlineStr">
+        <is>
+          <t>Desarrollo de soluciones de economía circular, reducción de residuos, reciclaje, ecodiseño y modelos de negocio circulares.</t>
+        </is>
+      </c>
+      <c r="W275" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X275" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y275" t="inlineStr">
+        <is>
+          <t>GIZ, KfW, universidades colombianas, gremios de recicladores y empresas de empaques.</t>
+        </is>
+      </c>
+      <c r="Z275" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AA275" t="inlineStr">
+        <is>
+          <t>Solicitar información adicional y preparar propuesta de idea.</t>
+        </is>
+      </c>
+      <c r="AB275" t="inlineStr">
+        <is>
+          <t>Contactar a IKI y solicitar guía de aplicación.</t>
+        </is>
+      </c>
+      <c r="AC275" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos</t>
+        </is>
+      </c>
+      <c r="AD275" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE275" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF275" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG275" t="inlineStr">
+        <is>
+          <t>No se dispone de fechas exactas; requiere verificación. | Fuente fuera del listado oficial conocido (international-climate-initiative.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH275" t="inlineStr">
+        <is>
+          <t>e2d2426ab3bef6f3</t>
+        </is>
+      </c>
+      <c r="AI275" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-09-25
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI275"/>
+  <dimension ref="A1:AI280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49088,6 +49088,891 @@
       <c r="AI275" t="inlineStr">
         <is>
           <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>VC-0275</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Convocatoria de inversión para pymes de economía circular, ingredientes naturales y agricultura sostenible</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Ingredientes naturales; agricultura sostenible</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Cofinanciación</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>USD 250,000</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N276" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q276" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R276" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/09/22/empresas-colombianas-podran-acceder-a-inversion-de-hasta-usd-250000-asi-puede-postularse</t>
+        </is>
+      </c>
+      <c r="S276" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T276" t="inlineStr">
+        <is>
+          <t>Convocatoria que seleccionará hasta 25 pymes colombianas vinculadas a ingredientes naturales, agricultura sostenible y economía circular, otorgándoles una inversión de hasta USD 250,000 y un proceso gratuito de 12 meses para preparar la atracción de capital.</t>
+        </is>
+      </c>
+      <c r="U276" t="inlineStr">
+        <is>
+          <t>Financia proyectos de economía circular y agricultura sostenible, alineados con los objetivos de cierre de ciclo de envases y ecodiseño de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V276" t="inlineStr">
+        <is>
+          <t>Desarrollo de envases reutilizables o reciclables; procesos de ecodiseño de empaques; integración de materiales bio‑basados; mejora de la cadena de valor de recicladores.</t>
+        </is>
+      </c>
+      <c r="W276" t="inlineStr">
+        <is>
+          <t>Ser pyme colombiana; operar en los sectores de ingredientes naturales, agricultura sostenible o economía circular; presentar plan de negocio y hoja de vida de la empresa.</t>
+        </is>
+      </c>
+      <c r="X276" t="inlineStr">
+        <is>
+          <t>Formulario de postulación; plan de negocio; estados financieros; certificaciones ambientales (si aplica).</t>
+        </is>
+      </c>
+      <c r="Y276" t="inlineStr">
+        <is>
+          <t>Cámaras de comercio; universidades con programas de ecodiseño; asociaciones de recicladores; entidades de apoyo a pymes como Bancóldex o iNNpulsa.</t>
+        </is>
+      </c>
+      <c r="Z276" t="inlineStr">
+        <is>
+          <t>Falta de información oficial sobre entidad financiadora y criterios de evaluación; posible requerimiento de co‑financiación que la pyme no pueda cubrir.</t>
+        </is>
+      </c>
+      <c r="AA276" t="inlineStr">
+        <is>
+          <t>Contactar a la fuente (Infobae) para confirmar entidad financiadora y obtener la guía oficial de postulación.</t>
+        </is>
+      </c>
+      <c r="AB276" t="inlineStr">
+        <is>
+          <t>Revisar la noticia completa, identificar la entidad responsable (posiblemente Bancóldex o Ministerio de Comercio) y solicitar los términos de referencia oficiales.</t>
+        </is>
+      </c>
+      <c r="AC276" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD276" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE276" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF276" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG276" t="inlineStr">
+        <is>
+          <t>La información proviene de un medio de noticias; no se encontró una página oficial de la convocatoria, por lo que se requiere verificación de la entidad financiadora y de los requisitos exactos. | Fuente fuera del listado oficial conocido (infobae.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH276" t="inlineStr">
+        <is>
+          <t>7b713f1ad66e8550</t>
+        </is>
+      </c>
+      <c r="AI276" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>VC-0276</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>CajaLab de Innovación de envases y empaques</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Conversápolis</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Colombia | América Latina</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Innovación en envases y empaques</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Piloto demostrativo; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N277" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P277" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R277" t="inlineStr">
+        <is>
+          <t>https://conversapolis.org/recurso/cajalab-de-innovacion</t>
+        </is>
+      </c>
+      <c r="S277" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T277" t="inlineStr">
+        <is>
+          <t>Convocatoria para proyectos de innovación en envases y empaques que contribuyan al desarrollo territorial sostenible, con financiamiento para iniciativas de desarrollo urbano.</t>
+        </is>
+      </c>
+      <c r="U277" t="inlineStr">
+        <is>
+          <t>Apoya la generación de soluciones circulares para envases y empaques, alineado con los objetivos de Visión Circular de la ANDI.</t>
+        </is>
+      </c>
+      <c r="V277" t="inlineStr">
+        <is>
+          <t>Desarrollo de materiales reciclables, ecodiseño, sistemas de recolección y reciclaje, inclusión de recicladores, modelos de negocio circulares.</t>
+        </is>
+      </c>
+      <c r="W277" t="inlineStr">
+        <is>
+          <t>Ser entidad colombiana o latinoamericana; presentar proyecto innovador; alineación con desarrollo territorial sostenible.</t>
+        </is>
+      </c>
+      <c r="X277" t="inlineStr">
+        <is>
+          <t>Propuesta técnica, plan financiero, certificaciones de entidad.</t>
+        </is>
+      </c>
+      <c r="Y277" t="inlineStr">
+        <is>
+          <t>Universidades, centros de investigación, asociaciones de recicladores, gremios de envases y empaques.</t>
+        </is>
+      </c>
+      <c r="Z277" t="inlineStr">
+        <is>
+          <t>Falta de claridad en montos y plazos; posible alta competencia.</t>
+        </is>
+      </c>
+      <c r="AA277" t="inlineStr">
+        <is>
+          <t>Revisar la convocatoria completa y preparar borrador de propuesta.</t>
+        </is>
+      </c>
+      <c r="AB277" t="inlineStr">
+        <is>
+          <t>Contactar a Conversápolis para solicitar términos de referencia y fechas exactas.</t>
+        </is>
+      </c>
+      <c r="AC277" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos</t>
+        </is>
+      </c>
+      <c r="AD277" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE277" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF277" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG277" t="inlineStr">
+        <is>
+          <t>Información limitada; se necesita confirmar apertura, fechas y montos específicos. | Fuente fuera del listado oficial conocido (conversapolis.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH277" t="inlineStr">
+        <is>
+          <t>23be55fb378583dd</t>
+        </is>
+      </c>
+      <c r="AI277" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>VC-0277</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>CircularEconomy 4Colombia Innovation Challenge</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>CircularEconomy 4Colombia (en colaboración con Agritech Challenge)</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Agri-food, empaques y reciclaje, ecodiseño, innovación</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Aceleración; Innovación</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N278" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P278" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R278" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S278" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T278" t="inlineStr">
+        <is>
+          <t>Challenge que busca acelerar soluciones circulares en el sector agroalimentario de Colombia, ofreciendo mentoría experta y potencial acceso a financiamiento o premios para proyectos que mejoren la circularidad de envases, residuos y procesos.</t>
+        </is>
+      </c>
+      <c r="U278" t="inlineStr">
+        <is>
+          <t>Relevante porque impulsa la economía circular en envases y empaques agroalimentarios, fomenta la inclusión de recicladores y la innovación sostenible.</t>
+        </is>
+      </c>
+      <c r="V278" t="inlineStr">
+        <is>
+          <t>Desarrollo de empaques reutilizables o reciclables; ecodiseño de productos agroalimentarios; modelos de negocio de reciclaje; inclusión de recicladores en la cadena de valor.</t>
+        </is>
+      </c>
+      <c r="W278" t="inlineStr">
+        <is>
+          <t>Ser empresa, startup o proyecto con sede en Colombia; presentar solución innovadora en economía circular para el sector agroalimentario.</t>
+        </is>
+      </c>
+      <c r="X278" t="inlineStr">
+        <is>
+          <t>Propuesta técnica, plan de negocio, evidencia de impacto ambiental.</t>
+        </is>
+      </c>
+      <c r="Y278" t="inlineStr">
+        <is>
+          <t>Gremios de envases, universidades de ingeniería, asociaciones de recicladores, Cámara de Comercio.</t>
+        </is>
+      </c>
+      <c r="Z278" t="inlineStr">
+        <is>
+          <t>Falta de claridad sobre montos y plazos; posible alta competencia.</t>
+        </is>
+      </c>
+      <c r="AA278" t="inlineStr">
+        <is>
+          <t>Revisar la convocatoria completa y preparar propuesta antes de la fecha límite.</t>
+        </is>
+      </c>
+      <c r="AB278" t="inlineStr">
+        <is>
+          <t>Acceder al sitio web, descargar bases de la convocatoria y contactar al organizador para confirmar fechas y requisitos.</t>
+        </is>
+      </c>
+      <c r="AC278" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AD278" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE278" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF278" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG278" t="inlineStr">
+        <is>
+          <t>Información de fechas, montos y requisitos exactos no disponible en la fuente; se necesita confirmar vigencia y condiciones. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH278" t="inlineStr">
+        <is>
+          <t>808de5d3d45d0699</t>
+        </is>
+      </c>
+      <c r="AI278" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>VC-0278</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Call for proposals to improve the circularity of multilayer flexible plastic food contact packaging</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>European Union (European Commission) – Horizon Europe / EU Funding Portal</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>European Union</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>UE y países asociados; terceros (p.ej. Colombia) pueden participar como socios en consorcio</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Plásticos flexibles – Envases multilayer de contacto alimentario</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Investigación aplicada; Innovación; Piloto demostrativo; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N279" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R279" t="inlineStr">
+        <is>
+          <t>https://eufundingportal.eu/call-for-proposals-to-improve-the-circularity-of-multilayer-flexible-plastic-food-contact-packaging-through-innovative-solutions</t>
+        </is>
+      </c>
+      <c r="S279" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T279" t="inlineStr">
+        <is>
+          <t>Financia proyectos de investigación y desarrollo que propongan soluciones innovadoras para aumentar la circularidad de envases flexibles multilayer de contacto alimentario, con énfasis en ecodiseño, reciclabilidad y escalamiento comercial. La convocatoria está dirigida a consorcios que incluyan al menos una entidad elegible de la UE y permite la participación de socios de terceros países como Colombia.</t>
+        </is>
+      </c>
+      <c r="U279" t="inlineStr">
+        <is>
+          <t>Relevante para Visión Circular porque aborda la circularidad de empaques plásticos flexibles, un foco clave de la agenda de cierre de ciclo de envases y reciclaje en Colombia.</t>
+        </is>
+      </c>
+      <c r="V279" t="inlineStr">
+        <is>
+          <t>Desarrollo de materiales reciclables; Ecodiseño de empaques multilayer; Tecnologías de separación y reciclaje; Pilotos de negocio para recolección y valorización de residuos de envases flexibles.</t>
+        </is>
+      </c>
+      <c r="W279" t="inlineStr">
+        <is>
+          <t>Formar un consorcio con al menos una entidad elegible de la UE; presentar propuesta técnica y financiera; cumplir con criterios de innovación y potencial de escalamiento; co‑financiación mínima requerida.</t>
+        </is>
+      </c>
+      <c r="X279" t="inlineStr">
+        <is>
+          <t>Formulario de propuesta, plan de trabajo, presupuesto detallado, cartas de intención de socios, evidencia de capacidad técnica.</t>
+        </is>
+      </c>
+      <c r="Y279" t="inlineStr">
+        <is>
+          <t>Universidades e institutos de investigación en Colombia (p.ej. Universidad Nacional, Universidad de los Andes); gremios de envases y empaques; asociaciones de recicladores; socios europeos especializados en materiales plásticos.</t>
+        </is>
+      </c>
+      <c r="Z279" t="inlineStr">
+        <is>
+          <t>Requisitos de co‑financiación; necesidad de socios europeos; cumplimiento de normas de la UE sobre plásticos de contacto alimentario.</t>
+        </is>
+      </c>
+      <c r="AA279" t="inlineStr">
+        <is>
+          <t>Iniciar contacto con la Oficina de Proyectos Internacionales de la UE para validar elegibilidad y explorar posibles socios europeos.</t>
+        </is>
+      </c>
+      <c r="AB279" t="inlineStr">
+        <is>
+          <t>Revisar la convocatoria completa en el portal EU Funding, elaborar una lista preliminar de socios europeos y preparar borrador de propuesta.</t>
+        </is>
+      </c>
+      <c r="AC279" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos internacionales / Alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD279" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE279" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF279" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG279" t="inlineStr">
+        <is>
+          <t>Se infiere que la convocatoria permite a entidades colombianas participar como socios, pero es necesario confirmar requisitos específicos de elegibilidad y fechas de apertura/cierre. | Fuente fuera del listado oficial conocido (eufundingportal.eu): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH279" t="inlineStr">
+        <is>
+          <t>2ab0abdcde825b59</t>
+        </is>
+      </c>
+      <c r="AI279" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>VC-0279</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>From Battery to Potential</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Inter‑American Development Bank (IDB)</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Internacional (América Latina y el Caribe)</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Colombia y demás países de América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Reciclaje y valorización de baterías; gestión de residuos de dispositivos electrónicos</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cooperación técnica; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/home/calls-proposals/battery-potential</t>
+        </is>
+      </c>
+      <c r="S280" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T280" t="inlineStr">
+        <is>
+          <t>Convocatoria abierta del IDB para financiar proyectos que fortalezcan la cadena de valor de baterías, desde la recolección y reciclaje hasta la generación de nuevos productos. Se busca impulsar soluciones innovadoras que reduzcan la huella ambiental y generen oportunidades de negocio en la región. Los fondos están dirigidos a entidades públicas, privadas y alianzas que demuestren viabilidad técnica y escalabilidad.</t>
+        </is>
+      </c>
+      <c r="U280" t="inlineStr">
+        <is>
+          <t>Apoya la visión de cerrar ciclos de materiales, fomenta la reutilización y reciclaje de baterías, y genera modelos de negocio circulares aplicables a la industria de envases y empaques.</t>
+        </is>
+      </c>
+      <c r="V280" t="inlineStr">
+        <is>
+          <t>Desarrollo de tecnologías de reciclaje de baterías; plataformas de recolección y logística inversa; ecodiseño de envases con componentes de baterías reutilizadas; inclusión de recicladores informales en la cadena de valor.</t>
+        </is>
+      </c>
+      <c r="W280" t="inlineStr">
+        <is>
+          <t>Ser organización con capacidad legal en un país elegible; presentar propuesta técnica y financiera; demostrar impacto ambiental y social; alianzas con actores locales (gremios, universidades, recicladores).</t>
+        </is>
+      </c>
+      <c r="X280" t="inlineStr">
+        <is>
+          <t>Formulario de aplicación; plan de trabajo; presupuesto detallado; evidencia de experiencia previa; cartas de apoyo de aliados locales.</t>
+        </is>
+      </c>
+      <c r="Y280" t="inlineStr">
+        <is>
+          <t>Cámaras de Industria, asociaciones de recicladores, universidades con programas de ingeniería de materiales, centros de investigación en energía y medio ambiente.</t>
+        </is>
+      </c>
+      <c r="Z280" t="inlineStr">
+        <is>
+          <t>Falta de claridad sobre montos y plazos; posible alta competencia; requisitos de cofinanciación no especificados.</t>
+        </is>
+      </c>
+      <c r="AA280" t="inlineStr">
+        <is>
+          <t>Revisar la convocatoria en detalle, contactar la oficina del IDB en Colombia para confirmar fechas y requisitos, y preparar una propuesta preliminar alineada con los objetivos de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB280" t="inlineStr">
+        <is>
+          <t>Acceder al portal del IDB, descargar la guía de aplicación y agendar una reunión interna con el equipo de alianzas para definir socios estratégicos.</t>
+        </is>
+      </c>
+      <c r="AC280" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y Alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD280" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE280" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF280" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG280" t="inlineStr">
+        <is>
+          <t>La página muestra la convocatoria pero no indica fechas de apertura o cierre; se asume que está activa por la ausencia de información de cierre. Se requiere confirmación directa con el IDB.</t>
+        </is>
+      </c>
+      <c r="AH280" t="inlineStr">
+        <is>
+          <t>dd4232645d0d6b42</t>
+        </is>
+      </c>
+      <c r="AI280" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-10-02
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI280"/>
+  <dimension ref="A1:AI288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45088,7 +45088,7 @@
       </c>
       <c r="N253" t="inlineStr">
         <is>
-          <t>Abierta permanentemente (según anuncio de lanzamiento)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="O253" t="inlineStr">
@@ -45193,7 +45193,7 @@
       </c>
       <c r="AI253" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -49973,6 +49973,1422 @@
       <c r="AI280" t="inlineStr">
         <is>
           <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>VC-0280</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>CircularEconomy 4Colombia – Agrichallenge</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Agricultura sostenible; Innovación agroalimentaria</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Innovación; Cofinanciación</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>Sí / Se espera cofinanciación del proyecto ganador</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/es/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S281" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T281" t="inlineStr">
+        <is>
+          <t>El Agrichallenge CircularEconomy 4Colombia busca soluciones innovadoras de economía circular aplicadas al sector agroalimentario colombiano. Ofrece mentoría, acceso a redes y posibles premios económicos a los proyectos seleccionados.</t>
+        </is>
+      </c>
+      <c r="U281" t="inlineStr">
+        <is>
+          <t>Fomenta la circularidad en la cadena agroalimentaria, alineado con los objetivos de cierre de ciclo, ecodiseño e inclusión de recicladores de Visión Circular de la ANDI.</t>
+        </is>
+      </c>
+      <c r="V281" t="inlineStr">
+        <is>
+          <t>Desarrollo de empaques biodegradables para productos agrícolas; sistemas de reutilización de residuos orgánicos; plataformas de logística circular para agroproductos.</t>
+        </is>
+      </c>
+      <c r="W281" t="inlineStr">
+        <is>
+          <t>Ser empresa, startup o proyecto colombiano; presentar solución innovadora en economía circular agro; cumplir con criterios de viabilidad y escalabilidad.</t>
+        </is>
+      </c>
+      <c r="X281" t="inlineStr">
+        <is>
+          <t>Formulario de inscripción, plan de negocio, evidencia de impacto circular, CV del equipo.</t>
+        </is>
+      </c>
+      <c r="Y281" t="inlineStr">
+        <is>
+          <t>Universidades agrícolas, centros de investigación, asociaciones de productores, recicladores de residuos orgánicos, incubadoras de innovación.</t>
+        </is>
+      </c>
+      <c r="Z281" t="inlineStr">
+        <is>
+          <t>Falta de claridad sobre montos y plazos; alta competencia; posible requerimiento de cofinanciación que no esté contemplado en el presupuesto interno.</t>
+        </is>
+      </c>
+      <c r="AA281" t="inlineStr">
+        <is>
+          <t>Revisar la página oficial, descargar la guía de postulación y preparar la documentación requerida antes de la fecha límite.</t>
+        </is>
+      </c>
+      <c r="AB281" t="inlineStr">
+        <is>
+          <t>Contactar al organizador vía correo disponible en la web para confirmar fechas de cierre, monto del premio y requisitos de cofinanciación.</t>
+        </is>
+      </c>
+      <c r="AC281" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AD281" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE281" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF281" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG281" t="inlineStr">
+        <is>
+          <t>Información limitada en la página; no se especifican fechas de apertura/cierre ni montos del premio. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH281" t="inlineStr">
+        <is>
+          <t>122c0b08650bc042</t>
+        </is>
+      </c>
+      <c r="AI281" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>VC-0281</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator Colombia – Call for Proposals 2026</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Climate Fin</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Economía baja en carbono</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>Asistencia técnica; Aceleración; Cofinanciación; Innovación</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>https://bogota.gov.co/boletin-oferta-internacional/climate-finance-accelerator-colombia-2026-acelera-proyectos-climatico</t>
+        </is>
+      </c>
+      <c r="S282" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T282" t="inlineStr">
+        <is>
+          <t>Convocatoria abierta por Climate Finance Accelerator Colombia 2026 para apoyar proyectos climáticos de alto impacto, proporcionando asistencia técnica, mentoría y acceso a potenciales inversores. La convocatoria está dirigida a iniciativas que fortalezcan su preparación para recibir inversión y escalar soluciones de transición a una economía baja en carbono.</t>
+        </is>
+      </c>
+      <c r="U282" t="inlineStr">
+        <is>
+          <t>Permite que proyectos de economía circular (reciclaje, ecodiseño, inclusión de recicladores) accedan a apoyo técnico y financiero para escalar sus soluciones climáticas.</t>
+        </is>
+      </c>
+      <c r="V282" t="inlineStr">
+        <is>
+          <t>Desarrollo de sistemas de reciclaje de envases; ecodiseño de empaques; modelos de negocio circulares; inclusión de recicladores informales; soluciones de gestión de residuos que reduzcan emisiones de GEI.</t>
+        </is>
+      </c>
+      <c r="W282" t="inlineStr">
+        <is>
+          <t>Presentar propuesta de proyecto climáticamente relevante; demostrar capacidad operativa y plan de negocio; alineación con objetivos de reducción de emisiones.</t>
+        </is>
+      </c>
+      <c r="X282" t="inlineStr">
+        <is>
+          <t>Formulario de propuesta; plan de trabajo; presupuesto detallado; evidencia de capacidad técnica y organizacional; certificaciones ambientales (si aplica).</t>
+        </is>
+      </c>
+      <c r="Y282" t="inlineStr">
+        <is>
+          <t>ANDI, gremios de envases y empaques, universidades con líneas de investigación en circularidad, asociaciones de recicladores, agencias de desarrollo regional.</t>
+        </is>
+      </c>
+      <c r="Z282" t="inlineStr">
+        <is>
+          <t>Falta de información pública sobre montos y fechas exactas; alta competencia; posible requerimiento de co‑financiación que las organizaciones pequeñas no puedan cubrir.</t>
+        </is>
+      </c>
+      <c r="AA282" t="inlineStr">
+        <is>
+          <t>Revisar la convocatoria en detalle, identificar criterios de elegibilidad y preparar una propuesta alineada a la economía circular.</t>
+        </is>
+      </c>
+      <c r="AB282" t="inlineStr">
+        <is>
+          <t>Acceder al portal oficial, descargar bases técnicas y calendario, y coordinar reunión interna para definir línea de proyecto y socios aliados.</t>
+        </is>
+      </c>
+      <c r="AC282" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AD282" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE282" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF282" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG282" t="inlineStr">
+        <is>
+          <t>La fuente no indica fechas de apertura/cierre ni montos disponibles; se asume que la convocatoria está abierta actualmente. Se requiere confirmar estos datos en la página oficial. | Fuente fuera del listado oficial conocido (bogota.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH282" t="inlineStr">
+        <is>
+          <t>fde8cba1f9c33c99</t>
+        </is>
+      </c>
+      <c r="AI282" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>VC-0282</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>CircularEconomy 4Colombia Innovation Challenge</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>CircularEconomy 4Colombia / Agritech Challenge</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Fundación</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Agri-food; Envases y empaques; Reciclaje</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Asistencia técnica; Innovación</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S283" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T283" t="inlineStr">
+        <is>
+          <t>Challenge que busca acelerar la transición a economía circular en el sector agroalimentario colombiano, ofreciendo mentoría experta y potenciales premios para soluciones innovadoras en envases, empaques y gestión de residuos.</t>
+        </is>
+      </c>
+      <c r="U283" t="inlineStr">
+        <is>
+          <t>Fomenta la circularidad en envases y empaques agroalimentarios, alineado con los objetivos de Visión Circular de ANDI.</t>
+        </is>
+      </c>
+      <c r="V283" t="inlineStr">
+        <is>
+          <t>Desarrollo de envases reutilizables, ecodiseño de empaques, sistemas de reciclaje de residuos agroalimentarios, inclusión de recicladores locales.</t>
+        </is>
+      </c>
+      <c r="W283" t="inlineStr">
+        <is>
+          <t>Ser empresa, startup o proyecto colombiano del sector agroalimentario; presentar solución innovadora; cumplir con criterios de circularidad.</t>
+        </is>
+      </c>
+      <c r="X283" t="inlineStr">
+        <is>
+          <t>Formulario de inscripción, plan de negocio, evidencia de impacto ambiental.</t>
+        </is>
+      </c>
+      <c r="Y283" t="inlineStr">
+        <is>
+          <t>Universidades agrícolas, centros de investigación, asociaciones de recicladores, cámaras de comercio.</t>
+        </is>
+      </c>
+      <c r="Z283" t="inlineStr">
+        <is>
+          <t>Posible cierre de convocatoria sin aviso; falta de claridad sobre montos de premio.</t>
+        </is>
+      </c>
+      <c r="AA283" t="inlineStr">
+        <is>
+          <t>Revisar la página oficial para confirmar fechas y requisitos; preparar propuesta de solución circular.</t>
+        </is>
+      </c>
+      <c r="AB283" t="inlineStr">
+        <is>
+          <t>Contactar a los organizadores vía formulario de consulta para obtener información actualizada.</t>
+        </is>
+      </c>
+      <c r="AC283" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AD283" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE283" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF283" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG283" t="inlineStr">
+        <is>
+          <t>Se infiere que la convocatoria está dirigida a soluciones de economía circular en agroalimentación; no se encontró información de fechas exactas. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH283" t="inlineStr">
+        <is>
+          <t>b75181bb9ce9de7d</t>
+        </is>
+      </c>
+      <c r="AI283" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>VC-0283</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Journalism Grants for Projects on Inclusive Recycling (Latin America)</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>International Journalists' Network (IJN)</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>ONG</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Latin America (incluye Colombia)</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Reciclaje</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Inclusión de recicladores; Comunicación y periodismo</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>US$4,500</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>https://ijnet.org/en/opportunity/journalism-grants-projects-inclusive-recycling-latin-america</t>
+        </is>
+      </c>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T284" t="inlineStr">
+        <is>
+          <t>Financia hasta US$4,500 a un proyecto periodístico que investigue y promueva el reciclaje inclusivo en América Latina, incluye mentoría individual y acceso a datos y casos de estudio. El proyecto debe entregarse en un máximo de dos meses.</t>
+        </is>
+      </c>
+      <c r="U284" t="inlineStr">
+        <is>
+          <t>Apoya la visibilidad y sensibilización sobre reciclaje inclusivo, alineado con los objetivos de inclusión de recicladores y economía circular de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V284" t="inlineStr">
+        <is>
+          <t>Investigación periodística sobre cadenas de reciclaje inclusivo; producción de reportajes o series multimedia; difusión de buenas prácticas de reciclaje en comunidades vulnerables.</t>
+        </is>
+      </c>
+      <c r="W284" t="inlineStr">
+        <is>
+          <t>Ser periodista o medio de comunicación; presentar descripción del proyecto y presupuesto detallado; compromiso de entregar resultados en 2 meses.</t>
+        </is>
+      </c>
+      <c r="X284" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto, CV o presentación del medio, presupuesto desglosado, plan de trabajo.</t>
+        </is>
+      </c>
+      <c r="Y284" t="inlineStr">
+        <is>
+          <t>Asociaciones de recicladores, universidades con programas de sostenibilidad, ONG ambientales, cámaras de comercio.</t>
+        </is>
+      </c>
+      <c r="Z284" t="inlineStr">
+        <is>
+          <t>Plazo corto y presupuesto limitado pueden restringir la profundidad del trabajo; necesidad de cumplir con requisitos de reporte.</t>
+        </is>
+      </c>
+      <c r="AA284" t="inlineStr">
+        <is>
+          <t>Revisar la convocatoria completa para confirmar fechas y requisitos, y preparar una propuesta enfocada en impacto social y ambiental.</t>
+        </is>
+      </c>
+      <c r="AB284" t="inlineStr">
+        <is>
+          <t>Acceder al enlace oficial, descargar la guía de aplicación y confirmar la fecha límite de presentación.</t>
+        </is>
+      </c>
+      <c r="AC284" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de comunicación y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD284" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE284" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF284" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG284" t="inlineStr">
+        <is>
+          <t>No se encontró la fecha de cierre en la información disponible; se asume que la convocatoria sigue abierta pero requiere confirmación. | Fuente fuera del listado oficial conocido (ijnet.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH284" t="inlineStr">
+        <is>
+          <t>6a530e314bbe228e</t>
+        </is>
+      </c>
+      <c r="AI284" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>VC-0284</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Circulate Capital Funding – Recycling Supply Chains</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Circulate Capital</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>EE.UU.</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Global; se aceptan propuestas de América Latina, incluyendo Colombia</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Cadenas de suministro de reciclaje; Upcycling; Digitalización</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Inversión; Aceleración</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>https://www.circulatecapital.com/apply-for-funding</t>
+        </is>
+      </c>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T285" t="inlineStr">
+        <is>
+          <t>Circulate Capital ofrece financiación a proyectos que fortalecen cadenas de suministro de reciclaje, incluyendo recolección, clasificación, upcycling y digitalización, mediante grants o inversión de capital. La convocatoria está abierta de forma continua y se evalúan propuestas de startups y empresas innovadoras.</t>
+        </is>
+      </c>
+      <c r="U285" t="inlineStr">
+        <is>
+          <t>Financia iniciativas de reciclaje y ecodiseño alineadas con los objetivos de cierre de ciclo de envases y empaques de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V285" t="inlineStr">
+        <is>
+          <t>Desarrollo de plataformas de trazabilidad; Tecnologías de clasificación de plásticos flexibles; Soluciones de upcycling para residuos de envases; Modelos de negocio de economía circular para PYMES.</t>
+        </is>
+      </c>
+      <c r="W285" t="inlineStr">
+        <is>
+          <t>Ser empresa o startup con solución innovadora en reciclaje; Operar en América Latina; Presentar plan de negocio y métricas de impacto.</t>
+        </is>
+      </c>
+      <c r="X285" t="inlineStr">
+        <is>
+          <t>Pitch deck; Plan de negocio; Evidencia de tracción; Información financiera.</t>
+        </is>
+      </c>
+      <c r="Y285" t="inlineStr">
+        <is>
+          <t>Universidades técnicas; Asociaciones de recicladores; Cámaras de comercio; Otros fondos de impacto.</t>
+        </is>
+      </c>
+      <c r="Z285" t="inlineStr">
+        <is>
+          <t>Falta de claridad sobre montos y criterios de elegibilidad; Competencia alta; Requisitos de cofinanciación no especificados.</t>
+        </is>
+      </c>
+      <c r="AA285" t="inlineStr">
+        <is>
+          <t>Revisar criterios detallados en la página, preparar pitch y contactar a Circulate Capital para validar elegibilidad de proyectos de envases.</t>
+        </is>
+      </c>
+      <c r="AB285" t="inlineStr">
+        <is>
+          <t>Designar equipo para elaborar pitch deck y agenda reunión preliminar con Circulate Capital antes del 15 de octubre.</t>
+        </is>
+      </c>
+      <c r="AC285" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de innovación y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD285" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE285" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF285" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG285" t="inlineStr">
+        <is>
+          <t>Se infiere que la convocatoria está abierta a nivel global; se necesita confirmar elegibilidad específica para Colombia y requisitos de cofinanciación.</t>
+        </is>
+      </c>
+      <c r="AH285" t="inlineStr">
+        <is>
+          <t>dc1bad14610e20ce</t>
+        </is>
+      </c>
+      <c r="AI285" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>VC-0285</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>SolNatura – Co‑funding Call for Proposals (Colombia)</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>International Climate Initiative (IKI) – Colombia</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Adaptación al cambio climático; Mitigación de emisiones; Conservación de biodiversidad</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>Cofinanciación; Grant no reembolsable</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>https://ikicolombia.com/en/solnatura-call-for-proposals-co-funding-for-projects-that-boost-climate-resilience-and-conservation-in-colombia</t>
+        </is>
+      </c>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T286" t="inlineStr">
+        <is>
+          <t>Convocatoria de co‑financiación para proyectos en Colombia que contribuyan a la resiliencia climática, mitigación de emisiones y conservación de ecosistemas. El financiamiento cubre parcialmente los costos elegibles bajo un esquema de co‑financiación con contrapartida local.</t>
+        </is>
+      </c>
+      <c r="U286" t="inlineStr">
+        <is>
+          <t>Aunque el foco principal es clima y biodiversidad, los proyectos pueden incluir componentes de economía circular como gestión de residuos, reciclaje y ecodiseño de empaques.</t>
+        </is>
+      </c>
+      <c r="V286" t="inlineStr">
+        <is>
+          <t>Gestión integral de residuos sólidos; Ecodiseño y reciclabilidad de envases; Modelos de negocio circulares para la cadena de valor de empaques; Inclusión de recicladores en la cadena de suministro.</t>
+        </is>
+      </c>
+      <c r="W286" t="inlineStr">
+        <is>
+          <t>Ser entidad colombiana (empresa, ONG, universidad, consorcio); presentar plan de proyecto con contrapartida financiera; alineación con los objetivos de adaptación, mitigación o biodiversidad.</t>
+        </is>
+      </c>
+      <c r="X286" t="inlineStr">
+        <is>
+          <t>Formulario de aplicación; propuesta técnica; presupuesto detallado; evidencia de contrapartida; certificaciones legales de la entidad.</t>
+        </is>
+      </c>
+      <c r="Y286" t="inlineStr">
+        <is>
+          <t>Gremios de la industria de empaques (ANDI, Cámara de Comercio), universidades con líneas de investigación en circularidad, asociaciones de recicladores, agencias de desarrollo regional.</t>
+        </is>
+      </c>
+      <c r="Z286" t="inlineStr">
+        <is>
+          <t>Falta de claridad sobre los criterios de evaluación específicos para economía circular; posible requerimiento de co‑financiación alta que limite la participación de pequeñas empresas.</t>
+        </is>
+      </c>
+      <c r="AA286" t="inlineStr">
+        <is>
+          <t>Revisar la guía de aplicación en la página de IKI, identificar proyectos internos que integren gestión de residuos o ecodiseño y preparar una propuesta preliminar con aliados estratégicos.</t>
+        </is>
+      </c>
+      <c r="AB286" t="inlineStr">
+        <is>
+          <t>Contactar a IKI Colombia para confirmar la ventana de presentación y solicitar el paquete de términos de referencia.</t>
+        </is>
+      </c>
+      <c r="AC286" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de Visión Circular / Alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD286" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE286" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF286" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG286" t="inlineStr">
+        <is>
+          <t>La convocatoria está activa según la página, pero no se indica fecha límite ni monto disponible; se requiere confirmar elegibilidad específica para proyectos de economía circular. | Fuente fuera del listado oficial conocido (ikicolombia.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH286" t="inlineStr">
+        <is>
+          <t>30664d9a123b7bb5</t>
+        </is>
+      </c>
+      <c r="AI286" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>VC-0286</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Advancing Circular Economy (ACE) Facility – Second Call for Proposals</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Caribbean Biodiversity Fund (CBF) – en colaboración con IDB Lab</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Caribe (regional)</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Países del Caribe y territorios elegibles (posible inclusión de Colombia – región Caribe)</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Reducción de contaminación marina; Innovación en empaques y plásticos; Inclusión de recicladores costeros</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Financiamiento climático; Cofinanciación</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>Sí / Descripción: se espera contrapartida local de los beneficiarios</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/posts/idblab_sargassum-coastalcommunities-environmental-activity-7285051949224198144-kyCw</t>
+        </is>
+      </c>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T287" t="inlineStr">
+        <is>
+          <t>Segunda convocatoria del ACE Facility que brinda financiamiento no reembolsable a proyectos innovadores de economía circular en el Caribe, enfocados en reducir la contaminación marina y promover la gestión sostenible de residuos, incluidos empaques plásticos.</t>
+        </is>
+      </c>
+      <c r="U287" t="inlineStr">
+        <is>
+          <t>Alta relevancia para Visión Circular al focalizarse en empaques, plásticos y modelos circulares que pueden ser replicados en la costa colombiana.</t>
+        </is>
+      </c>
+      <c r="V287" t="inlineStr">
+        <is>
+          <t>Desarrollo de sistemas de reciclaje de plásticos marinos; Ecodiseño de envases para reducir residuos costeros; Programas de inclusión de recicladores informales en la cadena de valor; Pilotos de economía circular en puertos y zonas costeras.</t>
+        </is>
+      </c>
+      <c r="W287" t="inlineStr">
+        <is>
+          <t>Ser entidad con sede en un país elegible del Caribe; presentar proyecto con impacto medible en reducción de residuos marinos; demostrar capacidad de ejecución y contrapartida financiera.</t>
+        </is>
+      </c>
+      <c r="X287" t="inlineStr">
+        <is>
+          <t>Formulario de aplicación; propuesta técnica; plan de monitoreo y evaluación; presupuesto; evidencia de contrapartida.</t>
+        </is>
+      </c>
+      <c r="Y287" t="inlineStr">
+        <is>
+          <t>Universidades costeras, ONG de gestión de residuos marinos, asociaciones de pescadores, cámaras de comercio de la región Caribe, entidades gubernamentales de medio ambiente.</t>
+        </is>
+      </c>
+      <c r="Z287" t="inlineStr">
+        <is>
+          <t>Posible exclusión de entidades colombianas si la convocatoria se limita estrictamente a países del Caribe; falta de información clara sobre montos y plazos.</t>
+        </is>
+      </c>
+      <c r="AA287" t="inlineStr">
+        <is>
+          <t>Verificar con CBF/IDB Lab la elegibilidad de organizaciones colombianas (especialmente de la zona Caribe) y solicitar el paquete de términos de referencia.</t>
+        </is>
+      </c>
+      <c r="AB287" t="inlineStr">
+        <is>
+          <t>Enviar correo de consulta a la dirección de contacto indicada en la publicación de LinkedIn para confirmar criterios de elegibilidad y fechas de presentación.</t>
+        </is>
+      </c>
+      <c r="AC287" t="inlineStr">
+        <is>
+          <t>Alianzas estratégicas / Relaciones institucionales</t>
+        </is>
+      </c>
+      <c r="AD287" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE287" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF287" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG287" t="inlineStr">
+        <is>
+          <t>La información proviene de una publicación en LinkedIn; no se dispone de una página oficial con detalle de la convocatoria, por lo que se necesita confirmar la vigencia y requisitos. | Fuente fuera del listado oficial conocido (linkedin.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH287" t="inlineStr">
+        <is>
+          <t>6002bd7d1e8fd0e7</t>
+        </is>
+      </c>
+      <c r="AI287" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>VC-0287</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>From Battery to Potential – Call for Proposals</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Inter‑American Development Bank (IDB)</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Banco multilateral</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Estados Unidos / América Latina</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Colombia y demás países de América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Reciclaje y reutilización de baterías; gestión de residuos de dispositivos electrónicos</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Sí / Descripción: se espera co‑financiación de los solicitantes o de socios estratégicos</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>2024-09-01</t>
+        </is>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>2024-10-31</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/home/calls-proposals/battery-potential</t>
+        </is>
+      </c>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T288" t="inlineStr">
+        <is>
+          <t>El IDB lanza una convocatoria para financiar proyectos que promuevan la reutilización, reciclaje y segunda vida de baterías, con el objetivo de reducir residuos y fomentar la economía circular en la región. Los proyectos deben presentar soluciones innovadoras y escalables y pueden recibir apoyo financiero no reembolsable.</t>
+        </is>
+      </c>
+      <c r="U288" t="inlineStr">
+        <is>
+          <t>Relevante porque aborda la gestión de residuos de baterías, un componente clave de la economía circular y la reducción de impactos ambientales en la cadena de valor de productos electrónicos.</t>
+        </is>
+      </c>
+      <c r="V288" t="inlineStr">
+        <is>
+          <t>Desarrollo de sistemas de recolección y reciclaje de baterías; diseño de productos con baterías de segunda vida; plataformas de logística inversa; modelos de negocio basados en la reutilización de energía almacenada.</t>
+        </is>
+      </c>
+      <c r="W288" t="inlineStr">
+        <is>
+          <t>Ser entidad legalmente constituida en Colombia o en otro país elegible; presentar proyecto con enfoque de innovación circular; demostrar capacidad técnica y financiera; co‑financiación mínima del 30 % del presupuesto total.</t>
+        </is>
+      </c>
+      <c r="X288" t="inlineStr">
+        <is>
+          <t>Formulario de aplicación en línea; plan de proyecto; presupuesto detallado; evidencia de co‑financiación; certificaciones de capacidad técnica.</t>
+        </is>
+      </c>
+      <c r="Y288" t="inlineStr">
+        <is>
+          <t>Universidades con programas de ingeniería eléctrica; asociaciones de recicladores; cámaras de comercio; ONG especializadas en gestión de residuos electrónicos.</t>
+        </is>
+      </c>
+      <c r="Z288" t="inlineStr">
+        <is>
+          <t>Posible alta competencia; requerimiento de co‑financiación que puede limitar la participación de pequeñas organizaciones; necesidad de cumplir con criterios de reporte financiero del IDB.</t>
+        </is>
+      </c>
+      <c r="AA288" t="inlineStr">
+        <is>
+          <t>Revisar la guía completa de la convocatoria y preparar una hoja de ruta de co‑financiación con potenciales aliados antes del 15 de octubre.</t>
+        </is>
+      </c>
+      <c r="AB288" t="inlineStr">
+        <is>
+          <t>Contactar al punto de atención del IDB (correo de la convocatoria) para confirmar requisitos de co‑financiación y solicitar aclaraciones sobre el monto disponible.</t>
+        </is>
+      </c>
+      <c r="AC288" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos de innovación y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD288" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE288" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF288" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG288" t="inlineStr">
+        <is>
+          <t>La información de monto disponible y criterios exactos de elegibilidad no está detallada en la página consultada; se asume que la convocatoria está abierta según la fecha de publicación del sitio.</t>
+        </is>
+      </c>
+      <c r="AH288" t="inlineStr">
+        <is>
+          <t>7e9843845b7dfc82</t>
+        </is>
+      </c>
+      <c r="AI288" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-10-09
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI288"/>
+  <dimension ref="A1:AI300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51389,6 +51389,2130 @@
       <c r="AI288" t="inlineStr">
         <is>
           <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>VC-0288</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia: Agrichallenge</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Agritech Challenge / Plataforma CircularEconomy4Colombia</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Agroindustria, valorización de biomasa y ecodiseño agroalimentario</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Innovación; Premio o challenge</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/es/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>Iniciativa de innovación abierta alineada con el Plan Nacional de Desarrollo 2022-2026 y metas de biodiversidad que busca catalizar soluciones circulares en la cadena agroalimentaria de Colombia. Ofrece acceso a mentores expertos, capacitación especializada y aceleración para fortalecer modelos de negocio sostenibles.</t>
+        </is>
+      </c>
+      <c r="U289" t="inlineStr">
+        <is>
+          <t>Permite explorar sinergias en el desarrollo de bioempaques, sustitución de materiales convencionales y aprovechamiento circular de flujos de subproductos en la agroindustria colombiana.</t>
+        </is>
+      </c>
+      <c r="V289" t="inlineStr">
+        <is>
+          <t>Pilotos de nuevos materiales y bioempaques; modelos circulares en cadenas de valor de alimentos y bebidas; valorización de residuos orgánicos.</t>
+        </is>
+      </c>
+      <c r="W289" t="inlineStr">
+        <is>
+          <t>Contar con soluciones innovadoras de economía circular aplicadas al sector agroalimentario en Colombia.</t>
+        </is>
+      </c>
+      <c r="X289" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y289" t="inlineStr">
+        <is>
+          <t>Empresas del sector agroindustrial afiliadas a la ANDI, centros de investigación, universidades y startups agritech.</t>
+        </is>
+      </c>
+      <c r="Z289" t="inlineStr">
+        <is>
+          <t>Posible enfoque centrado en etapas tempranas de aceleración con bajo componente de subvención en efectivo directa.</t>
+        </is>
+      </c>
+      <c r="AA289" t="inlineStr">
+        <is>
+          <t>Revisar los términos de referencia y fases del Agrichallenge para identificar si empresas de envases y empaques biobasados pueden postular o si Visión Circular puede articularse como aliado mentor/institucional.</t>
+        </is>
+      </c>
+      <c r="AB289" t="inlineStr">
+        <is>
+          <t>Ingresar a la plataforma oficial para revisar las fechas de corte vigentes y los beneficios específicos del programa.</t>
+        </is>
+      </c>
+      <c r="AC289" t="inlineStr">
+        <is>
+          <t>Coordinación de Innovación y Proyectos</t>
+        </is>
+      </c>
+      <c r="AD289" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE289" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF289" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG289" t="inlineStr">
+        <is>
+          <t>La vinculación a metas del PND y COP16 sugiere respaldo institucional multilateral o gubernamental, aunque el monto exacto de capital semilla no se desglosa en el extracto. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH289" t="inlineStr">
+        <is>
+          <t>114fe699575b45c5</t>
+        </is>
+      </c>
+      <c r="AI289" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>VC-0289</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Premio de Economía Circular del Cauca 2026</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Urbaser Popayán y Zona Franca del Cauca</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Colombia (departamento del Cauca / iniciativas regionales)</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Gestión de residuos, valorización territorial e impacto social</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/UrbaserPopayan/posts/-ya-est%C3%A1n-abiertas-las-postulaciones-al-premio-de-econom%C3%ADa-circular-del-cauca-20/1586606226812732</t>
+        </is>
+      </c>
+      <c r="S290" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T290" t="inlineStr">
+        <is>
+          <t>Convocatoria territorial dirigida a organizaciones con iniciativas implementadas de economía circular que cuenten con resultados verificables y generación de valor ambiental, social o económico. Busca premiar y visibilizar buenas prácticas empresariales y comunitarias en el departamento del Cauca.</t>
+        </is>
+      </c>
+      <c r="U290" t="inlineStr">
+        <is>
+          <t>Permite visibilizar y articular iniciativas territoriales de aprovechamiento de residuos, empresas locales de la cadena de empaques y asociaciones de recicladores de oficio en el suroccidente del país.</t>
+        </is>
+      </c>
+      <c r="V290" t="inlineStr">
+        <is>
+          <t>Modelos de economía circular territorial; esquemas de inclusión y reconocimiento a la gestión de recicladores; pilotos de aprovechamiento empresarial en zonas francas.</t>
+        </is>
+      </c>
+      <c r="W290" t="inlineStr">
+        <is>
+          <t>Iniciativas en marcha con resultados verificables en el departamento del Cauca con impacto social, ambiental o económico.</t>
+        </is>
+      </c>
+      <c r="X290" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y290" t="inlineStr">
+        <is>
+          <t>Urbaser, Zona Franca del Cauca, empresas afiliadas a ANDI Seccional Cauca y asociaciones de recicladores locales.</t>
+        </is>
+      </c>
+      <c r="Z290" t="inlineStr">
+        <is>
+          <t>Alcance geográfico restringido al Cauca y posible falta de dotación monetaria significativa si se trata principalmente de reconocimiento honorífico.</t>
+        </is>
+      </c>
+      <c r="AA290" t="inlineStr">
+        <is>
+          <t>Verificar con Urbaser Popayán o Zona Franca del Cauca la fecha límite exacta y los incentivos del premio para postular casos de éxito vinculados al programa Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB290" t="inlineStr">
+        <is>
+          <t>Contactar a los organizadores para acceder a los términos de referencia oficiales y verificar si el cierre está vigente.</t>
+        </is>
+      </c>
+      <c r="AC290" t="inlineStr">
+        <is>
+          <t>Coordinación Territorial / Alianzas</t>
+        </is>
+      </c>
+      <c r="AD290" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE290" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF290" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG290" t="inlineStr">
+        <is>
+          <t>El texto de la publicación está cortado ('hasta el 6...'), por lo que no es posible determinar con certeza el día y mes exacto de cierre sin ingresar al formulario oficial. | Fuente fuera del listado oficial conocido (facebook.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH290" t="inlineStr">
+        <is>
+          <t>b415666831cef2fb</t>
+        </is>
+      </c>
+      <c r="AI290" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>VC-0290</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Programa AECID de Cooperación Triangular - Modelos de Economía Circular en Entidades Públicas (Lote 22)</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Agencia Española de Cooperación Internacional para el Desarrollo (AECID)</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Colombia y países de América Latina</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Modelos de economía circular en entidades públicas y gestión territorial</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>https://www.asocapitales.co/sites/default/files/files/technical_documents/boletin-cooperacion-internacional-julio-2026.pdf</t>
+        </is>
+      </c>
+      <c r="S291" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T291" t="inlineStr">
+        <is>
+          <t>Programa orientado a estructurar y transferir modelos de economía circular aplicados en entidades públicas a través del esquema de Cooperación Triangular de la AECID. Busca fortalecer capacidades técnicas, operativas y de política pública local en gestión circular.</t>
+        </is>
+      </c>
+      <c r="U291" t="inlineStr">
+        <is>
+          <t>Permite posicionar el modelo de Visión Circular ANDI ante entidades públicas territoriales (ciudades capitales), promoviendo marcos regulatorios favorables para el cumplimiento REP y modelos de aprovechamiento colaborativo de envases y empaques.</t>
+        </is>
+      </c>
+      <c r="V291" t="inlineStr">
+        <is>
+          <t>Estructuración de pilotos de economía circular territorial, articulación público-privada para la separación en la fuente y esquemas de recolección diferenciada con municipios.</t>
+        </is>
+      </c>
+      <c r="W291" t="inlineStr">
+        <is>
+          <t>Articulación con entidades públicas o Gobiernos locales (asociados a Asocapitales/AECID) bajo la modalidad de Cooperación Triangular.</t>
+        </is>
+      </c>
+      <c r="X291" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y291" t="inlineStr">
+        <is>
+          <t>Asocapitales, alcaldías de ciudades capitales, ministerios sectoriales y AECID Colombia.</t>
+        </is>
+      </c>
+      <c r="Z291" t="inlineStr">
+        <is>
+          <t>Restricción de postulación exclusiva a entidades de carácter público o necesidad obligatoria de consorcio público-privado liderado por el sector gubernamental.</t>
+        </is>
+      </c>
+      <c r="AA291" t="inlineStr">
+        <is>
+          <t>Contactar al equipo de cooperación de Asocapitales para confirmar los términos de referencia específicos del Lote 22 y evaluar si Visión Circular ANDI puede participar como socio implementador técnico privado.</t>
+        </is>
+      </c>
+      <c r="AB291" t="inlineStr">
+        <is>
+          <t>Descargar y revisar las bases completas del boletín de Asocapitales y solicitar reunión de alineación con el área técnica de sostenibilidad y cooperación de dicha entidad.</t>
+        </is>
+      </c>
+      <c r="AC291" t="inlineStr">
+        <is>
+          <t>Coordinación de Alianzas y Cooperación / Gerencia de Visión Circular</t>
+        </is>
+      </c>
+      <c r="AD291" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE291" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF291" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG291" t="inlineStr">
+        <is>
+          <t>El boletín de Asocapitales cita fecha límite 06/07/2026 y titula el boletín como julio de 2026; esto podría corresponder a un error de digitación por parte de Asocapitales (posiblemente 2024 o 2025) o a una ventana de programación plurianual. | Fuente fuera del listado oficial conocido (asocapitales.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH291" t="inlineStr">
+        <is>
+          <t>31c0fa5c41e9309d</t>
+        </is>
+      </c>
+      <c r="AI291" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>VC-0291</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator Colombia – Call for Proposals 2026</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator (CFA)</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Mitigación del cambio climático y transición baja en carbono</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>https://bogota.gov.co/boletin-oferta-internacional/climate-finance-accelerator-colombia-2026-acelera-proyectos-climatico</t>
+        </is>
+      </c>
+      <c r="S292" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>Convocatoria abierta para apoyar proyectos climáticos de alto impacto en Colombia en su preparación para recibir inversión. Busca acelerar iniciativas que aporten a la transición hacia una economía baja en carbono mediante asistencia técnica para estructuración financiera y vinculación con inversionistas.</t>
+        </is>
+      </c>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>Es pertinente para estructurar y escalar proyectos o modelos de negocio circulares de empresas aliadas a Visión Circular que generen mitigación verificable de emisiones (ej. valorización y reciclaje a gran escala) y requieran bancabilidad.</t>
+        </is>
+      </c>
+      <c r="V292" t="inlineStr">
+        <is>
+          <t>Escalamiento de infraestructura de aprovechamiento y reciclaje de plásticos; modelos circulares corporativos con reducción comprobada de GEI; encadenamientos productivos de circularidad con viabilidad de inversión privada.</t>
+        </is>
+      </c>
+      <c r="W292" t="inlineStr">
+        <is>
+          <t>Proyectos climáticos de alto impacto con potencial de reducción de carbono que busquen financiamiento o inversión para su escalamiento.</t>
+        </is>
+      </c>
+      <c r="X292" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y292" t="inlineStr">
+        <is>
+          <t>Empresas transformadoras del programa Visión Circular, fondos de inversión de impacto, banca comercial y de desarrollo.</t>
+        </is>
+      </c>
+      <c r="Z292" t="inlineStr">
+        <is>
+          <t>CFA tradicionalmente opera como aceleradora de preparación para la inversión y conexión con inversionistas (debt/equity), no como un fondo de grant no reembolsable directo; puede exigir montos mínimos de capital proyectado elevados.</t>
+        </is>
+      </c>
+      <c r="AA292" t="inlineStr">
+        <is>
+          <t>Ingresar a la nota técnica de la Alcaldía Mayor de Bogotá para consultar los términos de referencia, el enlace directo al portal de aplicación de CFA y la fecha límite de recepción de postulaciones.</t>
+        </is>
+      </c>
+      <c r="AB292" t="inlineStr">
+        <is>
+          <t>Descargar y analizar los términos de referencia detallados para verificar si iniciativas de reciclaje de envases y empaques cumplen con el umbral de mitigación y tamaño de inversión requerido.</t>
+        </is>
+      </c>
+      <c r="AC292" t="inlineStr">
+        <is>
+          <t>Coordinación de Atracción de Inversión y Proyectos Especiales</t>
+        </is>
+      </c>
+      <c r="AD292" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE292" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF292" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG292" t="inlineStr">
+        <is>
+          <t>Inferido: El programa suele estar respaldado por la cooperación del Reino Unido (UK PACT). Aunque se enfoca en clima general, los proyectos de economía circular orientados al desvío masivo de residuos e industrialización de reciclaje suelen calificar bajo metas de mitigación de carbono. | Fuente fuera del listado oficial conocido (bogota.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH292" t="inlineStr">
+        <is>
+          <t>d5495f170f752f4a</t>
+        </is>
+      </c>
+      <c r="AI292" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>VC-0292</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Convocatoria regional para soluciones innovadoras en plásticos en Colombia, Chile y México</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Cempre Colombia, WRAP y Red Global de Pactos por los Plásticos</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>ONG</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Colombia / Reino Unido</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Colombia, Chile y México</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Envases y empaques</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Gestión sostenible de envases y empaques plásticos</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>Hasta USD 10.000 por solución seleccionada (bolsa para 10 soluciones)</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>https://www.pactoglobal-colombia.org/news/convocatoria-regional-otorgara-hasta-usd-10-000-a-soluciones-innovadoras-en-plasticos-en-colombia-chile-y-mexico.html</t>
+        </is>
+      </c>
+      <c r="S293" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>Convocatoria regional impulsada por Cempre, WRAP y la Red Global de Pactos por los Plásticos que seleccionará 10 soluciones empresariales innovadoras enfocadas en mejorar la gestión sostenible de envases y empaques plásticos en Colombia, México y Chile. El programa otorga hasta USD 10.000 a iniciativas destacadas para apalancar su implementación y escalamiento.</t>
+        </is>
+      </c>
+      <c r="U293" t="inlineStr">
+        <is>
+          <t>Alineación directa con los objetivos de Visión Circular ANDI, al enfocarse explícitamente en soluciones de economía circular y cierre de ciclo para envases y empaques plásticos en Colombia.</t>
+        </is>
+      </c>
+      <c r="V293" t="inlineStr">
+        <is>
+          <t>Pilotos empresariales de ecodiseño, modelos de aprovechamiento y reciclaje de plásticos posconsumo, soluciones para plásticos de difícil reciclabilidad y nuevos esquemas circulares de empaque.</t>
+        </is>
+      </c>
+      <c r="W293" t="inlineStr">
+        <is>
+          <t>Soluciones empresariales innovadoras aplicables a la cadena de valor de envases y empaques plásticos en los países objetivo.</t>
+        </is>
+      </c>
+      <c r="X293" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y293" t="inlineStr">
+        <is>
+          <t>Empresas afiliadas a Visión Circular ANDI, transformadores y recicladores de plástico, Pacto por los Plásticos, Cempre Colombia.</t>
+        </is>
+      </c>
+      <c r="Z293" t="inlineStr">
+        <is>
+          <t>Monto unitario acotado (hasta USD 10.000), enfocado en etapas tempranas o pilotos específicos; alta competencia regional.</t>
+        </is>
+      </c>
+      <c r="AA293" t="inlineStr">
+        <is>
+          <t>Contactar de inmediato al equipo de Cempre Colombia y Pacto Global Red Colombia para obtener los términos de referencia vigentes y la fecha límite exacta tras la ampliación de la convocatoria.</t>
+        </is>
+      </c>
+      <c r="AB293" t="inlineStr">
+        <is>
+          <t>Descargar las bases completas desde el enlace de Pacto Global Colombia y perfilar 1 o 2 pilotos empresariales de empresas vinculadas a Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AC293" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos e Innovación / Alianzas</t>
+        </is>
+      </c>
+      <c r="AD293" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE293" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF293" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG293" t="inlineStr">
+        <is>
+          <t>El artículo reporta una ampliación de la convocatoria regional. Se infiere que el proceso sigue activo, pero requiere validar con urgencia la nueva fecha de cierre. | Fuente fuera del listado oficial conocido (pactoglobal-colombia.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH293" t="inlineStr">
+        <is>
+          <t>6aa4b5b93069382a</t>
+        </is>
+      </c>
+      <c r="AI293" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>VC-0293</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia Innovation Challenge</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>AgriTech Challenge (consorcio de innovación y aceleración)</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Sector agroalimentario, valorización de residuos y modelos circulares</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Aceleración; Asistencia técnica; Innovación</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S294" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>Desafío de innovación diseñado para acelerar la transición hacia una economía circular en el sector agroalimentario de Colombia, alineado con el Plan Nacional de Desarrollo 2022-2026 y la COP16. Ofrece a las soluciones seleccionadas acceso a mentorías de expertos, acompañamiento técnico integral y escalamiento de modelos circulares.</t>
+        </is>
+      </c>
+      <c r="U294" t="inlineStr">
+        <is>
+          <t>Altamente relevante para Visión Circular ANDI en el impulso de empaques sostenibles, bioempaques, valorización de subproductos y encadenamientos de economía circular con la industria de alimentos y bebidas.</t>
+        </is>
+      </c>
+      <c r="V294" t="inlineStr">
+        <is>
+          <t>Pilotos de nuevos materiales/bioplásticos para empaques agroindustriales; aprovechamiento y valorización de mermas y residuos agropecuarios; ecodiseño y logística inversa de envases del sector agroalimentario.</t>
+        </is>
+      </c>
+      <c r="W294" t="inlineStr">
+        <is>
+          <t>Soluciones e innovaciones orientadas a la economía circular aplicables al sector agroalimentario colombiano.</t>
+        </is>
+      </c>
+      <c r="X294" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y294" t="inlineStr">
+        <is>
+          <t>Empresas del sector agroindustrial y de alimentos de la ANDI, centros de investigación, universidades y startups bio/circulares.</t>
+        </is>
+      </c>
+      <c r="Z294" t="inlineStr">
+        <is>
+          <t>Falta visibilidad inmediata en el extracto de los términos de referencia, montos en efectivo y cronograma detallado de postulaciones.</t>
+        </is>
+      </c>
+      <c r="AA294" t="inlineStr">
+        <is>
+          <t>Ingresar al portal web oficial para corroborar el estado actual de la convocatoria, bases del concurso, fechas límites y determinar si aplica para empresas vinculadas a ANDI o consorcios de innovación.</t>
+        </is>
+      </c>
+      <c r="AB294" t="inlineStr">
+        <is>
+          <t>Revisar la URL oficial (agritechchallenge.org) y contactar a los organizadores para validar si el periodo de postulaciones continúa abierto o si contempla una segunda cohorte.</t>
+        </is>
+      </c>
+      <c r="AC294" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos e innovación</t>
+        </is>
+      </c>
+      <c r="AD294" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE294" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF294" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG294" t="inlineStr">
+        <is>
+          <t>El reto está directamente articulado con metas de Colombia y la agenda de la CBD COP16. Se infiere que incluye aceleración técnica y mentoría especializada. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH294" t="inlineStr">
+        <is>
+          <t>9b0caa7f7bd2426e</t>
+        </is>
+      </c>
+      <c r="AI294" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>VC-0294</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator (CFA) Colombia</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Climate Finance Accelerator (CFA)</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Residuos y economía circular (waste and circular economy)</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>Aceleración; Asistencia técnica; Financiamiento climático</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>USD 1M a USD 30M</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>https://www.climatefinanceaccelerator.com/countries/colombia</t>
+        </is>
+      </c>
+      <c r="S295" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>El Climate Finance Accelerator (CFA) apoya proyectos climáticos en Colombia en etapas desde generación temprana de ingresos hasta escalamiento, incluyendo una línea prioritaria en residuos y economía circular. Facilita asistencia técnica y vinculación con inversionistas para proyectos con necesidades de capital entre USD 1M y USD 30M.</t>
+        </is>
+      </c>
+      <c r="U295" t="inlineStr">
+        <is>
+          <t>Directamente alineada con Visión Circular ANDI al contar con un eje enfocado en residuos y economía circular para escalar proyectos empresariales y modelos de negocio de alto impacto.</t>
+        </is>
+      </c>
+      <c r="V295" t="inlineStr">
+        <is>
+          <t>Escalamiento de infraestructura de aprovechamiento y reciclaje de envases y empaques, plantas de valorización de plásticos flexibles, y modelos de negocio circulares empresariales.</t>
+        </is>
+      </c>
+      <c r="W295" t="inlineStr">
+        <is>
+          <t>Proyectos en sectores priorizados (AFOLU, energías renovables, residuos y economía circular) con madurez de negocio demostrable y requerimientos financieros entre USD 1M y USD 30M.</t>
+        </is>
+      </c>
+      <c r="X295" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y295" t="inlineStr">
+        <is>
+          <t>Empresas afiliadas a Visión Circular ANDI, transformadores y recicladores industriales, fondos de inversión de impacto y banca de desarrollo.</t>
+        </is>
+      </c>
+      <c r="Z295" t="inlineStr">
+        <is>
+          <t>La página web reseña los proyectos de la cohorte ya seleccionada; es necesario verificar si la convocatoria para una nueva cohorte está abierta o en planeación.</t>
+        </is>
+      </c>
+      <c r="AA295" t="inlineStr">
+        <is>
+          <t>Contactar al equipo del CFA Colombia mediante el formulario/contacto de su portal para indagar fechas de apertura de la siguiente cohorte y postular proyectos del pipeline de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AB295" t="inlineStr">
+        <is>
+          <t>Enviar consulta formal al punto de contacto de CFA Colombia para conocer el cronograma de postulaciones de la próxima ronda.</t>
+        </is>
+      </c>
+      <c r="AC295" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos y Atracción de Recursos</t>
+        </is>
+      </c>
+      <c r="AD295" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE295" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF295" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG295" t="inlineStr">
+        <is>
+          <t>Se infiere que el programa opera por ciclos periódicos de cohortes. Dado que el extracto reporta proyectos ya seleccionados, se clasifica para verificación activa de apertura. | Fuente fuera del listado oficial conocido (climatefinanceaccelerator.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH295" t="inlineStr">
+        <is>
+          <t>619a63281d46b569</t>
+        </is>
+      </c>
+      <c r="AI295" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>VC-0295</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>HORIZON-CL6-2026-01-CIRCBIO-01: Improving circularity of multilayer flexible plastic food contact packaging</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Comisión Europea (Horizon Europe)</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Estados miembros de la UE, países asociados y terceros países elegibles en consorcio (incluye Colombia)</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Envases y empaques</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Plásticos flexibles</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Investigación aplicada; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R296" t="inlineStr">
+        <is>
+          <t>https://fasi.eu/en/grants/6c3f8bd1-dca9-39a4-97be-2508f8072e55</t>
+        </is>
+      </c>
+      <c r="S296" t="inlineStr">
+        <is>
+          <t>https://atomgrants.com/grant/improving-circularity-multilayer-flexible-plastic-food-contact-packaging-european-commission</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>Financia proyectos colaborativos orientados a desarrollar y demostrar soluciones circulares y de reciclaje avanzado para envases plásticos flexibles multicapa en contacto con alimentos. Busca integrar innovaciones físicas y digitales para superar barreras técnicas de reciclabilidad.</t>
+        </is>
+      </c>
+      <c r="U296" t="inlineStr">
+        <is>
+          <t>Es de máxima prioridad técnica, pues aborda plásticos flexibles y multicapa en contacto con alimentos, uno de los mayores desafíos para el cierre de ciclo y cumplimiento de metas REP de las empresas de la ANDI.</t>
+        </is>
+      </c>
+      <c r="V296" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje químico/mecánico avanzado de empaques flexibles multicapa; pruebas de ecodiseño y sustitución de barreras; validación de trazabilidad digital en cadenas de posconsumo.</t>
+        </is>
+      </c>
+      <c r="W296" t="inlineStr">
+        <is>
+          <t>Conformación obligatoria de consorcios internacionales con entidades de países europeos elegibles; enfoque en innovación y demostración tecnológica.</t>
+        </is>
+      </c>
+      <c r="X296" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y296" t="inlineStr">
+        <is>
+          <t>Centros tecnológicos y universidades europeas y colombianas, transformadores de plástico, empresas de alimentos y bebidas de la ANDI.</t>
+        </is>
+      </c>
+      <c r="Z296" t="inlineStr">
+        <is>
+          <t>Complejidad técnica y administrativa de Horizon Europe; Colombia participa como tercer país, por lo que se requiere validar si aplica a financiación directa de la UE o requiere cofinanciación nacional/en especie.</t>
+        </is>
+      </c>
+      <c r="AA296" t="inlineStr">
+        <is>
+          <t>Rastrear el tópico oficial en el 'EU Funding &amp; Tenders Portal' para confirmar el texto final de la convocatoria 2026 e identificar redes o consorcios europeos en formación.</t>
+        </is>
+      </c>
+      <c r="AB296" t="inlineStr">
+        <is>
+          <t>Contactar puntos nacionales de contacto (NCP) de Horizon Europe en Colombia o redes universitarias aliadas para monitorear apertura del call CIRCBIO 2026.</t>
+        </is>
+      </c>
+      <c r="AC296" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos e Innovación / Alianzas Internacionales</t>
+        </is>
+      </c>
+      <c r="AD296" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE296" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF296" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG296" t="inlineStr">
+        <is>
+          <t>Se infiere que Colombia puede participar bajo el esquema estándar de Horizon Europe para terceros países en consorcios transnacionales. | Fuente fuera del listado oficial conocido (fasi.eu): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH296" t="inlineStr">
+        <is>
+          <t>9fcebddb1feb21e7</t>
+        </is>
+      </c>
+      <c r="AI296" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>VC-0296</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Catalytic Green Fund - Driving Decarbonization in Latin America and the Caribbean</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>BID Lab (Banco Interamericano de Desarrollo)</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (incluye Colombia)</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Descarbonización, modelos de negocio circulares e innovación tecnológica</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Cofinanciación; Asistencia técnica; Innovación; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R297" t="inlineStr">
+        <is>
+          <t>https://bidlab.org/en/news/new-call-proposals-catalytic-green-fund-driving-decarbonization-latin-america-and-caribbean</t>
+        </is>
+      </c>
+      <c r="S297" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>Convocatoria lanzada por BID Lab dirigida a Organizaciones de Apoyo al Emprendimiento (ESOs), tales como aceleradoras, cámaras de comercio, gremios, universidades y fundaciones. Financia e impulsa proyectos e innovaciones tecnológicas orientadas a mitigar emisiones de GEI y acelerar la transición hacia la economía circular.</t>
+        </is>
+      </c>
+      <c r="U297" t="inlineStr">
+        <is>
+          <t>Muy alta relevancia, ya que la ANDI y Visión Circular actúan como organizaciones articuladoras del ecosistema productivo capaces de estructurar programas de aceleración o escalamiento de tecnologías circulares y de aprovechamiento de envases.</t>
+        </is>
+      </c>
+      <c r="V297" t="inlineStr">
+        <is>
+          <t>Aceleración de soluciones de ecodiseño y plásticos flexibles; escalamiento de modelos de logística inversa y trazabilidad REP; pilotos empresariales de sustitución de materiales.</t>
+        </is>
+      </c>
+      <c r="W297" t="inlineStr">
+        <is>
+          <t>Ser una Organización de Apoyo al Emprendimiento (ESO) o entidad del ecosistema de innovación con capacidad operativa en América Latina y el Caribe.</t>
+        </is>
+      </c>
+      <c r="X297" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y297" t="inlineStr">
+        <is>
+          <t>Universidades, cámaras de comercio aliadas, aceleradoras corporativas y empresas miembro de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="Z297" t="inlineStr">
+        <is>
+          <t>Exigencia probable de contrapartida institucional y alta competencia regional entre entidades intermediarias.</t>
+        </is>
+      </c>
+      <c r="AA297" t="inlineStr">
+        <is>
+          <t>Descargar y analizar la guía operativa en el portal de BID Lab para contrastar los requerimientos de contrapartida y fechas límites.</t>
+        </is>
+      </c>
+      <c r="AB297" t="inlineStr">
+        <is>
+          <t>Revisar los términos de referencia detallados en bidlab.org y definir el rol de Visión Circular/ANDI como entidad postulante principal.</t>
+        </is>
+      </c>
+      <c r="AC297" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos y Alianzas</t>
+        </is>
+      </c>
+      <c r="AD297" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE297" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF297" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG297" t="inlineStr">
+        <is>
+          <t>El perfil encaja de forma precisa en el rol gremial e intermediario de la ANDI como entidad promotora de innovación empresarial circular.</t>
+        </is>
+      </c>
+      <c r="AH297" t="inlineStr">
+        <is>
+          <t>7243cf96633a073e</t>
+        </is>
+      </c>
+      <c r="AI297" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>VC-0297</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>SolNatura Call for Proposals: Co-funding for projects that boost climate resilience and conservation in Colombia</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Iniciativa Internacional del Clima (IKI Colombia)</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Alemania / Colombia</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Resiliencia climática, conservación y sostenibilidad territorial</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cofinanciación</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr">
+        <is>
+          <t>2024-10-28</t>
+        </is>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr">
+        <is>
+          <t>https://ikicolombia.com/en/solnatura-call-for-proposals-co-funding-for-projects-that-boost-climate-resilience-and-conservation-in-colombia</t>
+        </is>
+      </c>
+      <c r="S298" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>Fondo de cofinanciación para proyectos en Colombia orientados a incrementar la resiliencia climática y promover la conservación de ecosistemas, abierto desde el 28 de octubre de 2024.</t>
+        </is>
+      </c>
+      <c r="U298" t="inlineStr">
+        <is>
+          <t>Relevancia indirecta para iniciativas de economía circular territorial donde el manejo adecuado de residuos y empaques mitiga la presión sobre ecosistemas y fuentes hídricas estratégicas.</t>
+        </is>
+      </c>
+      <c r="V298" t="inlineStr">
+        <is>
+          <t>Modelos de economía circular comunitaria y territorial en zonas de amortiguamiento ambiental; prevención de contaminación plástica en cuencas hidrográficas.</t>
+        </is>
+      </c>
+      <c r="W298" t="inlineStr">
+        <is>
+          <t>Proyectos ejecutados en territorio colombiano que demuestren impacto en resiliencia climática y conservación.</t>
+        </is>
+      </c>
+      <c r="X298" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y298" t="inlineStr">
+        <is>
+          <t>Organizaciones territoriales, ONG ambientales, autoridades ambientales y asociaciones de recicladores en municipios priorizados.</t>
+        </is>
+      </c>
+      <c r="Z298" t="inlineStr">
+        <is>
+          <t>El núcleo temático está orientado principalmente a conservación biológica y soluciones basadas en la naturaleza, por lo que una propuesta de circularidad debe fundamentar fuertemente su beneficio ecológico.</t>
+        </is>
+      </c>
+      <c r="AA298" t="inlineStr">
+        <is>
+          <t>Acceder a las bases de la convocatoria en ikicolombia.com para constatar la fecha límite y si admite componentes de economía circular territorial.</t>
+        </is>
+      </c>
+      <c r="AB298" t="inlineStr">
+        <is>
+          <t>Verificar en ikicolombia.com la elegibilidad técnica de proyectos de residuos y la ventana de cierre.</t>
+        </is>
+      </c>
+      <c r="AC298" t="inlineStr">
+        <is>
+          <t>Coordinación de Alianzas y Cooperación Internacional</t>
+        </is>
+      </c>
+      <c r="AD298" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE298" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF298" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG298" t="inlineStr">
+        <is>
+          <t>Apertura registrada el 28 de octubre de 2024. Su viabilidad depende de estructurar la propuesta bajo un ángulo de reducción de impactos antropogénicos y resiliencia climática. | Fuente fuera del listado oficial conocido (ikicolombia.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH298" t="inlineStr">
+        <is>
+          <t>f10bc4d1938bc5a5</t>
+        </is>
+      </c>
+      <c r="AI298" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>VC-0298</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>GEF SGP CSO Challenge Program</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) / Unión Internacional para la Conservación de la Naturaleza (UICN)</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Suiza / Estados Unidos</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Países beneficiarios del GEF / SGP (incluye Colombia y América Latina)</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Sostenibilidad ambiental</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Escalamiento de innovaciones ambientales comunitarias e inclusión</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Asistencia técnica; Escalamiento; Innovación</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>Hasta 300,000 USD por proyecto (fondo global de USD 10 millones)</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>Próxima apertura</t>
+        </is>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>https://iucn.org/press-release/202510/new-gef-programme-set-deliver-grants-usd-300000-civil-society-led</t>
+        </is>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>Iniciativa del GEF Small Grants Programme ejecutada por UICN que otorgará subvenciones competitivas de hasta 300.000 USD a organizaciones de la sociedad civil (OSC). Su objetivo es financiar y brindar asistencia técnica para escalar soluciones ambientales innovadoras lideradas a nivel local.</t>
+        </is>
+      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>Permite estructurar modelos de economía circular comunitaria y proyectos de inclusión socioeconómica de recicladores de base y gestores locales de residuos, articulados con fundaciones empresariales o el brazo social de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V299" t="inlineStr">
+        <is>
+          <t>Escalamiento de centros locales de acopio y clasificación de empaques; fortalecimiento de asociaciones de recicladores en ecodiseño y aprovechamiento; iniciativas comunitarias de prevención de plásticos y residuos.</t>
+        </is>
+      </c>
+      <c r="W299" t="inlineStr">
+        <is>
+          <t>Dirigido a organizaciones de la sociedad civil (OSC), comunidades locales, mujeres y jóvenes. Los proyectos deben demostrar innovación ambiental y potencial de réplica o escalamiento.</t>
+        </is>
+      </c>
+      <c r="X299" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y299" t="inlineStr">
+        <is>
+          <t>Fundaciones empresariales vinculadas a la ANDI, asociaciones territoriales de recicladores de oficio, ONG ambientales colombianas acreditadas ante UICN/GEF.</t>
+        </is>
+      </c>
+      <c r="Z299" t="inlineStr">
+        <is>
+          <t>Elegibilidad directa restringida a entidades de la sociedad civil (requiere presentarse mediante o en consorcio con una OSC/Fundación); competencia a nivel global.</t>
+        </is>
+      </c>
+      <c r="AA299" t="inlineStr">
+        <is>
+          <t>Monitorear el portal de UICN y del GEF SGP para acceder a los lineamientos operativos y la apertura formal de la ventana de postulación.</t>
+        </is>
+      </c>
+      <c r="AB299" t="inlineStr">
+        <is>
+          <t>Contactar a la oficina del GEF SGP en Colombia (PNUD/UICN) y preparar un banco de iniciativas de economía circular de base comunitaria con fundaciones aliadas.</t>
+        </is>
+      </c>
+      <c r="AC299" t="inlineStr">
+        <is>
+          <t>Coordinación de Alianzas y Cooperación Internacional</t>
+        </is>
+      </c>
+      <c r="AD299" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE299" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF299" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG299" t="inlineStr">
+        <is>
+          <t>Se infiere que Colombia será elegible por ser país receptor activo del GEF y del SGP. La fecha formal de cierre aún no ha sido publicada en los comunicados de lanzamiento. | Fuente fuera del listado oficial conocido (iucn.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH299" t="inlineStr">
+        <is>
+          <t>95272639cea8cae9</t>
+        </is>
+      </c>
+      <c r="AI299" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>VC-0299</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Programme (SGP)</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF) – implementado por UNDP, FAO y Conservation International</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Multilateral</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>127 países incluidos, entre ellos Colombia</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Gestión de residuos; Innovación comunitaria; Ecodiseño</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Asistencia técnica; Cooperación técnica</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R300" t="inlineStr">
+        <is>
+          <t>https://www.cepf.net/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S300" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T300" t="inlineStr">
+        <is>
+          <t>El GEF Small Grants Programme financia proyectos de innovación comunitaria y desarrollo de capacidad en áreas ambientales, incluyendo gestión de residuos y economía circular. Otorga subvenciones no reembolsables a organizaciones locales para implementar soluciones piloto.</t>
+        </is>
+      </c>
+      <c r="U300" t="inlineStr">
+        <is>
+          <t>Apoya iniciativas de reciclaje, ecodiseño y cierre de ciclo de envases, alineadas con los objetivos de Visión Circular de la ANDI.</t>
+        </is>
+      </c>
+      <c r="V300" t="inlineStr">
+        <is>
+          <t>Pilotos de reciclaje de plásticos flexibles; Programas de inclusión de recicladores; Desarrollo de empaques reutilizables; Capacitación en ecodiseño.</t>
+        </is>
+      </c>
+      <c r="W300" t="inlineStr">
+        <is>
+          <t>Ser organización sin ánimo de lucro, entidad comunitaria o asociación; proyecto enfocado en gestión de residuos o economía circular; presencia en país elegible.</t>
+        </is>
+      </c>
+      <c r="X300" t="inlineStr">
+        <is>
+          <t>Propuesta técnica, presupuesto, evidencia de capacidad organizacional, cartas de apoyo.</t>
+        </is>
+      </c>
+      <c r="Y300" t="inlineStr">
+        <is>
+          <t>Gremios de recicladores, universidades, centros de investigación, cámaras de comercio.</t>
+        </is>
+      </c>
+      <c r="Z300" t="inlineStr">
+        <is>
+          <t>Competencia alta; requisitos de cofinanciación pueden variar; plazos no claros.</t>
+        </is>
+      </c>
+      <c r="AA300" t="inlineStr">
+        <is>
+          <t>Revisar la guía de aplicación del SGP y preparar una propuesta preliminar enfocada en reciclaje de envases.</t>
+        </is>
+      </c>
+      <c r="AB300" t="inlineStr">
+        <is>
+          <t>Contactar al punto focal del GEF en Colombia para confirmar fechas de convocatoria y requisitos específicos.</t>
+        </is>
+      </c>
+      <c r="AC300" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD300" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE300" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF300" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG300" t="inlineStr">
+        <is>
+          <t>La página indica que el programa está activo, pero no se especifican fechas de apertura o cierre ni montos concretos; se requiere confirmar que haya una convocatoria abierta para 2024. | Fuente fuera del listado oficial conocido (cepf.net): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH300" t="inlineStr">
+        <is>
+          <t>a74b70c02ff70300</t>
+        </is>
+      </c>
+      <c r="AI300" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-10-16
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI300"/>
+  <dimension ref="A1:AI304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45088,7 +45088,7 @@
       </c>
       <c r="N253" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Abierta permanentemente</t>
         </is>
       </c>
       <c r="O253" t="inlineStr">
@@ -45193,7 +45193,7 @@
       </c>
       <c r="AI253" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -47566,7 +47566,7 @@
       </c>
       <c r="N267" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Abierta permanentemente</t>
         </is>
       </c>
       <c r="O267" t="inlineStr">
@@ -47656,7 +47656,7 @@
       </c>
       <c r="AF267" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AG267" t="inlineStr">
@@ -47671,7 +47671,7 @@
       </c>
       <c r="AI267" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -53513,6 +53513,714 @@
       <c r="AI300" t="inlineStr">
         <is>
           <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>VC-0300</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>AECID – Cooperación Triangular – Modelos de Economía Circular en Entidades Públicas (Lote 22)</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Agencia Española de Cooperación Internacional para el Desarrollo (AECID)</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Colombia y otros países de América Latina elegibles bajo modalidad triangular</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>Modelos de economía circular en entidades públicas</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cooperación técnica</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>Sí / Descripción: se espera cofinanciación de la entidad beneficiaria o de socios locales</t>
+        </is>
+      </c>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R301" t="inlineStr">
+        <is>
+          <t>https://www.asocapitales.co/sites/default/files/files/technical_documents/boletin-cooperacion-internacional-julio-2026.pdf</t>
+        </is>
+      </c>
+      <c r="S301" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T301" t="inlineStr">
+        <is>
+          <t>Convocatoria de la AECID para financiar proyectos que desarrollen y escalen modelos de economía circular en entidades públicas de Colombia y la región. El apoyo cubre asistencia técnica, desarrollo de pilotos y actividades de transferencia de conocimiento.</t>
+        </is>
+      </c>
+      <c r="U301" t="inlineStr">
+        <is>
+          <t>Financia la generación de modelos circulares que pueden ser replicados por empresas y gremios, alineado con los objetivos de cierre de ciclo de envases y empaques de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V301" t="inlineStr">
+        <is>
+          <t>Diseño e implementación de sistemas de reciclaje de envases; desarrollo de plataformas de trazabilidad; fortalecimiento de la cadena de valor de plásticos flexibles; inclusión de recicladores informales en procesos públicos.</t>
+        </is>
+      </c>
+      <c r="W301" t="inlineStr">
+        <is>
+          <t>Ser entidad pública o consorcio público‑privado; presentar proyecto con impacto territorial; demostrar capacidad técnica y plan de sostenibilidad.</t>
+        </is>
+      </c>
+      <c r="X301" t="inlineStr">
+        <is>
+          <t>Formulario de aplicación, plan de proyecto, presupuesto, evidencia de capacidad institucional, cartas de apoyo de socios locales.</t>
+        </is>
+      </c>
+      <c r="Y301" t="inlineStr">
+        <is>
+          <t>Ministerio de Ambiente y Desarrollo Sostenible, Cámaras de Comercio, universidades (p.ej. Universidad Nacional), asociaciones de recicladores, ANDI y sus gremios sectoriales.</t>
+        </is>
+      </c>
+      <c r="Z301" t="inlineStr">
+        <is>
+          <t>Posible restricción a entidades exclusivamente públicas; requerimiento de cofinanciación que podría limitar la participación de pequeñas empresas.</t>
+        </is>
+      </c>
+      <c r="AA301" t="inlineStr">
+        <is>
+          <t>Evaluar la posibilidad de presentar una propuesta conjunta entre una entidad pública y un consorcio liderado por ANDI para cumplir con el requisito de entidad pública.</t>
+        </is>
+      </c>
+      <c r="AB301" t="inlineStr">
+        <is>
+          <t>Descargar la guía completa del llamado (página 5 del PDF) y organizar una reunión interna con el área de alianzas para definir socios públicos potenciales.</t>
+        </is>
+      </c>
+      <c r="AC301" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos y Alianzas Estratégicas</t>
+        </is>
+      </c>
+      <c r="AD301" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE301" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF301" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG301" t="inlineStr">
+        <is>
+          <t>La convocatoria está dirigida a entidades públicas; la elegibilidad de consorcios público‑privados no está clara y requiere confirmación. | Fuente fuera del listado oficial conocido (asocapitales.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH301" t="inlineStr">
+        <is>
+          <t>4e4dc0a50474580b</t>
+        </is>
+      </c>
+      <c r="AI301" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>VC-0301</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Convocatoria Visión Circular ANDI 2024</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Asociación Nacional de Industriales (ANDI)</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>Envases y empaques; Modelos de negocio circulares</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cooperación técnica</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/VisionCircularANDI/photos/impulsamos-la-innovaci%C3%B3n-sostenible-visi%C3%B3n-circular-andi-abre-convocatoria-para-/592199606985664</t>
+        </is>
+      </c>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T302" t="inlineStr">
+        <is>
+          <t>ANDI abre una convocatoria para financiar proyectos que transformen el futuro de los empaques y envases mediante modelos de economía circular. Se busca apoyar iniciativas de ecodiseño, reutilización, inclusión de recicladores y cumplimiento de la REP.</t>
+        </is>
+      </c>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>Alta, porque la convocatoria está alineada directamente con los objetivos de Visión Circular de impulsar la circularidad de envases y empaques en Colombia.</t>
+        </is>
+      </c>
+      <c r="V302" t="inlineStr">
+        <is>
+          <t>Desarrollo de empaques reutilizables; ecodiseño de envases; integración de recicladores formales e informales; soluciones de trazabilidad y cumplimiento de la REP.</t>
+        </is>
+      </c>
+      <c r="W302" t="inlineStr">
+        <is>
+          <t>Ser empresa, gremio, universidad o entidad colombiana; presentar proyecto alineado con economía circular de envases; cumplir con los criterios de innovación y viabilidad.</t>
+        </is>
+      </c>
+      <c r="X302" t="inlineStr">
+        <is>
+          <t>Propuesta técnica; plan de negocio; evidencia de capacidad operativa; certificaciones ambientales (si aplica).</t>
+        </is>
+      </c>
+      <c r="Y302" t="inlineStr">
+        <is>
+          <t>Universidades, centros de investigación, asociaciones de recicladores, incubadoras de negocio.</t>
+        </is>
+      </c>
+      <c r="Z302" t="inlineStr">
+        <is>
+          <t>Falta de información pública sobre montos, plazos y criterios de evaluación; posible alta competencia.</t>
+        </is>
+      </c>
+      <c r="AA302" t="inlineStr">
+        <is>
+          <t>Contactar a ANDI a través del mensaje de la publicación para solicitar la guía oficial de la convocatoria y los términos de referencia.</t>
+        </is>
+      </c>
+      <c r="AB302" t="inlineStr">
+        <is>
+          <t>Enviar correo o mensaje a la cuenta de Facebook indicada solicitando el documento de bases y condiciones.</t>
+        </is>
+      </c>
+      <c r="AC302" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas estratégicas</t>
+        </is>
+      </c>
+      <c r="AD302" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE302" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF302" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG302" t="inlineStr">
+        <is>
+          <t>Información limitada en la publicación; se necesita confirmar fechas de cierre, montos y requisitos específicos. | Fuente fuera del listado oficial conocido (facebook.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH302" t="inlineStr">
+        <is>
+          <t>f0d7e46b9a2b9593</t>
+        </is>
+      </c>
+      <c r="AI302" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>VC-0302</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Secure Bio-based Packaging Funding: HORIZON-JU-CBE-2023-IAFlag-03</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>European Commission – Horizon Europe</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Unión Europea y países asociados (incl. Colombia como tercer país mediante consorcio)</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>Bio-based packaging, envases y empaques</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>Hasta 17,000,000 EUR por proyecto</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N303" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R303" t="inlineStr">
+        <is>
+          <t>https://www.grantbite.com/en/funding/horizon-bio-packaging-circularity-funding</t>
+        </is>
+      </c>
+      <c r="S303" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T303" t="inlineStr">
+        <is>
+          <t>Financia proyectos de innovación en envases bio‑basados para acelerar la transición a una economía circular. Se otorgan hasta 17 millones de euros por proyecto bajo la modalidad de Acción de Innovación.</t>
+        </is>
+      </c>
+      <c r="U303" t="inlineStr">
+        <is>
+          <t>Apoya el desarrollo de envases sostenibles y la circularidad de plásticos, alineado con los objetivos de Visión Circular de la ANDI.</t>
+        </is>
+      </c>
+      <c r="V303" t="inlineStr">
+        <is>
+          <t>Desarrollo de materiales bio‑basados; diseño ecológico de empaques; pruebas piloto de reciclabilidad; integración de recicladores en la cadena de valor.</t>
+        </is>
+      </c>
+      <c r="W303" t="inlineStr">
+        <is>
+          <t>Consorcio con al menos una entidad elegible de la UE; proyecto de 3 años; enfoque innovador; cumplimiento de criterios de circularidad.</t>
+        </is>
+      </c>
+      <c r="X303" t="inlineStr">
+        <is>
+          <t>Formulario de propuesta Horizon Europe; plan de trabajo; presupuesto; cartas de intención de socios.</t>
+        </is>
+      </c>
+      <c r="Y303" t="inlineStr">
+        <is>
+          <t>Universidades colombianas; centros de investigación; asociaciones de recicladores; empresas de empaques; Cámara de Comercio de Bogotá.</t>
+        </is>
+      </c>
+      <c r="Z303" t="inlineStr">
+        <is>
+          <t>Necesidad de socios europeos; cumplimiento de requisitos administrativos de Horizon; alta competencia.</t>
+        </is>
+      </c>
+      <c r="AA303" t="inlineStr">
+        <is>
+          <t>Iniciar contacto con la Oficina de Proyectos Internacionales de la UE y buscar socios europeos.</t>
+        </is>
+      </c>
+      <c r="AB303" t="inlineStr">
+        <is>
+          <t>Revisar guía de participación de terceros países y preparar borrador de consorcio.</t>
+        </is>
+      </c>
+      <c r="AC303" t="inlineStr">
+        <is>
+          <t>Coordinación de Alianzas Estratégicas</t>
+        </is>
+      </c>
+      <c r="AD303" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE303" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF303" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG303" t="inlineStr">
+        <is>
+          <t>La convocatoria parece activa, pero la fecha límite no está disponible en la información extraída; se requiere confirmar vigencia y elegibilidad de Colombia. | Fuente fuera del listado oficial conocido (grantbite.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH303" t="inlineStr">
+        <is>
+          <t>95bc93ca581801d4</t>
+        </is>
+      </c>
+      <c r="AI303" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>VC-0303</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Catalytic Green Fund – Driving Decarbonization in Latin America and the Caribbean</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>IDB Lab (Inter-American Development Bank)</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Países de América Latina y el Caribe, incluido Colombia</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Descarbonización, innovación circular, gestión de residuos</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cofinanciación; Asistencia técnica; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>Sí / Descripción: se espera co‑financiación de socios locales o regionales</t>
+        </is>
+      </c>
+      <c r="N304" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>https://bidlab.org/en/news/new-call-proposals-catalytic-green-fund-driving-decarbonization-latin-america-and-caribbean</t>
+        </is>
+      </c>
+      <c r="S304" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T304" t="inlineStr">
+        <is>
+          <t>El Catalytic Green Fund busca financiar a Organizaciones de Apoyo al Emprendedor (ESOs) que impulsen proyectos y tecnologías que reduzcan emisiones de GEI y promuevan la economía circular en la región. El apoyo incluye fondos no reembolsables, co‑financiación y asistencia técnica para escalar soluciones innovadoras.</t>
+        </is>
+      </c>
+      <c r="U304" t="inlineStr">
+        <is>
+          <t>Financia proyectos de economía circular y gestión de residuos, alineados con los objetivos de Visión Circular de ANDI para envases, reciclaje e inclusión de recicladores.</t>
+        </is>
+      </c>
+      <c r="V304" t="inlineStr">
+        <is>
+          <t>Desarrollo de soluciones de reciclaje de envases; ecodiseño de empaques; plataformas de inclusión de recicladores; modelos de negocio circulares para plásticos flexibles; pruebas piloto de tecnologías de reutilización.</t>
+        </is>
+      </c>
+      <c r="W304" t="inlineStr">
+        <is>
+          <t>Ser una Organización de Apoyo al Emprendedor (ej. cámara de comercio, aceleradora, universidad, fondo de impacto) con presencia en LAC; presentar proyecto con impacto medible en descarbonización y circularidad.</t>
+        </is>
+      </c>
+      <c r="X304" t="inlineStr">
+        <is>
+          <t>Formulario de propuesta, plan de negocio, evidencia de capacidad operativa, presupuesto detallado, cartas de apoyo de socios locales.</t>
+        </is>
+      </c>
+      <c r="Y304" t="inlineStr">
+        <is>
+          <t>Cámaras de comercio (ANDI), universidades (Universidad Nacional de Colombia), asociaciones de recicladores, fundaciones de innovación, fondos de inversión de impacto.</t>
+        </is>
+      </c>
+      <c r="Z304" t="inlineStr">
+        <is>
+          <t>Posible cierre de la convocatoria antes de la fecha de revisión; requerimiento de co‑financiación que podría limitar la participación si no se asegura el aporte local.</t>
+        </is>
+      </c>
+      <c r="AA304" t="inlineStr">
+        <is>
+          <t>Contactar a IDB Lab para confirmar estado de la convocatoria y requisitos de elegibilidad específicos para ANDI como cámara sectorial.</t>
+        </is>
+      </c>
+      <c r="AB304" t="inlineStr">
+        <is>
+          <t>Revisar la guía completa de la convocatoria en la URL oficial, preparar borrador de proyecto alineado con los criterios y solicitar reunión preliminar con IDB Lab.</t>
+        </is>
+      </c>
+      <c r="AC304" t="inlineStr">
+        <is>
+          <t>Coordinación de Alianzas Estratégicas y Proyectos de Innovación</t>
+        </is>
+      </c>
+      <c r="AD304" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE304" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF304" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG304" t="inlineStr">
+        <is>
+          <t>No se encontraron fechas de apertura/cierre en la fuente; se asume que la convocatoria está abierta o próxima a abrir según la publicación reciente.</t>
+        </is>
+      </c>
+      <c r="AH304" t="inlineStr">
+        <is>
+          <t>725c4a313ce893dd</t>
+        </is>
+      </c>
+      <c r="AI304" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: oportunidades Visión Circular 2026-10-23
</commit_message>
<xml_diff>
--- a/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
+++ b/funding-agent/data/oportunidades_atraccion_recursos_vision_circular.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI304"/>
+  <dimension ref="A1:AI323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22609,12 +22609,12 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>Lanzado (según noticia del GEF)</t>
+          <t>Recientemente lanzado en Colombia</t>
         </is>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (programa abierto permanentemente en ciclos)</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -22689,7 +22689,7 @@
       </c>
       <c r="AD126" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AE126" t="inlineStr">
@@ -22714,7 +22714,7 @@
       </c>
       <c r="AI126" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -46963,7 +46963,7 @@
       </c>
       <c r="AI263" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -50301,19 +50301,19 @@
       </c>
       <c r="AD282" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE282" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF282" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AE282" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AF282" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AG282" t="inlineStr">
         <is>
           <t>La fuente no indica fechas de apertura/cierre ni montos disponibles; se asume que la convocatoria está abierta actualmente. Se requiere confirmar estos datos en la página oficial. | Fuente fuera del listado oficial conocido (bogota.gov.co): verificar oficialidad</t>
@@ -50326,7 +50326,7 @@
       </c>
       <c r="AI282" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -51894,19 +51894,19 @@
       </c>
       <c r="AD291" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE291" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF291" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AE291" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AF291" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AG291" t="inlineStr">
         <is>
           <t>El boletín de Asocapitales cita fecha límite 06/07/2026 y titula el boletín como julio de 2026; esto podría corresponder a un error de digitación por parte de Asocapitales (posiblemente 2024 o 2025) o a una ventana de programación plurianual. | Fuente fuera del listado oficial conocido (asocapitales.co): verificar oficialidad</t>
@@ -51919,7 +51919,7 @@
       </c>
       <c r="AI291" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -54221,6 +54221,3369 @@
       <c r="AI304" t="inlineStr">
         <is>
           <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>VC-0304</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia: Agrichallenge</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Agritech Challenge (plataforma de innovación agroalimentaria)</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Colombia / Internacional</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Colombia (énfasis en sector agroalimentario)</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Innovación agroalimentaria, cierre de ciclo, reducción de residuos agrícolas</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Aceleración; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R305" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/es/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S305" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T305" t="inlineStr">
+        <is>
+          <t>Challenge de innovación CircularEconomy4Colombia diseñado para catalizar soluciones de economía circular en el sector agroalimentario colombiano. Ofrece acceso a mentores expertos y capacitación para emprendedores y empresas innovadoras. Alineado con el Plan Nacional de Desarrollo 2022-2026 de Colombia y objetivos de la COP 16 (CBD).</t>
+        </is>
+      </c>
+      <c r="U305" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: busca soluciones de economía circular, cierre de ciclo de residuos y modelos de negocio circulares en sector agroalimentario, con potencial para envases/empaques agrícolas, reciclabilidad y ecodiseño.</t>
+        </is>
+      </c>
+      <c r="V305" t="inlineStr">
+        <is>
+          <t>Soluciones de cierre de ciclo en cadena agroalimentaria; Ecodiseño de empaques agrícolas; Reciclaje y aprovechamiento de residuos agrícolas; Modelos de negocio circulares territoriales; Inclusión de pequeños productores en economía circular.</t>
+        </is>
+      </c>
+      <c r="W305" t="inlineStr">
+        <is>
+          <t>No especificado (inferencia: probablemente solución innovadora en economía circular, equipo constituido, alineación con objetivos nacionales).</t>
+        </is>
+      </c>
+      <c r="X305" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y305" t="inlineStr">
+        <is>
+          <t>Gremios agroindustriales (Andi, ANDI sectorial), universidades con programas de agroindustria, centros tecnológicos especializados en agroecología y sostenibilidad, recicladores organizados, cooperativas agrícolas.</t>
+        </is>
+      </c>
+      <c r="Z305" t="inlineStr">
+        <is>
+          <t>No especificado si hay restricciones de etapa empresarial, tamaño de empresa o sector específico dentro de agroalimentario. Requiere verificación de elegibilidad para pequeñas empresas y recicladores organizados.</t>
+        </is>
+      </c>
+      <c r="AA305" t="inlineStr">
+        <is>
+          <t>Contactar directamente a Agritech Challenge para obtener bases detalladas, montos y cronograma exacto. Identificar 2-3 soluciones piloto del portafolio de Visión Circular que apliquen a agroalimentario. Articular con gremios afiliados a ANDI en sector agrícola.</t>
+        </is>
+      </c>
+      <c r="AB305" t="inlineStr">
+        <is>
+          <t>1) Verificar bases de convocatoria y estado actual en agritechchallenge.org; 2) Revisar si hay integración con instituciones de cooperación (bilateral, multilateral) que fortalezcan el prize pool; 3) Mapear empresas/emprendimientos de Visión Circular elegibles; 4) Preparar pitch 1-2 meses antes de cierre (si no se conoce fecha exacta).</t>
+        </is>
+      </c>
+      <c r="AC305" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos e Innovación; Alianzas Estratégicas; Equipo de Pilotos Empresariales.</t>
+        </is>
+      </c>
+      <c r="AD305" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE305" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF305" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG305" t="inlineStr">
+        <is>
+          <t>Challenge activo, alineado con políticas nacionales. No se especifica monto, pero oferta de mentorías y capacitación tiene valor intangible relevante. Inferencia: probablemente abierta actualmente (se menciona Plan 2022-2026 y COP 16 Colombia 2024 como contexto). Requiere verificación de dates y elegibilidad de tipo de soluciones. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH305" t="inlineStr">
+        <is>
+          <t>9bffe99f036bfc66</t>
+        </is>
+      </c>
+      <c r="AI305" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>VC-0305</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Premio de Economía Circular del Cauca 2026</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Urbaser (empresa de gestión de residuos / Autoridad o entidad regional del Cauca)</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Gobierno | Otro (empresa privada con responsabilidad social)</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Colombia (Departamento del Cauca)</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Colombia (Cauca)</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>Iniciativas de economía circular, reciclaje, gestión de residuos territorial</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Reconocimiento; Posible cofinanciación</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N306" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>2026-04-08 (fecha de cierre según fuente Facebook; VIGENTE HOY)</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr">
+        <is>
+          <t>https://urbaser.co/premio-economia-circular</t>
+        </is>
+      </c>
+      <c r="S306" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/UrbaserPopayan/posts/hoy-cierra-la-convocatoria-hasta-el-final-del-d%C3%ADa-podr%C3%A1s-postular-tu-iniciativa-/1600533042086717</t>
+        </is>
+      </c>
+      <c r="T306" t="inlineStr">
+        <is>
+          <t>Premio regional de Economía Circular del Cauca 2026 convocado por Urbaser. Está CERRANDO HOY (2026-04-08) con plazo hasta fin de día para postulaciones. Busca reconocer iniciativas innovadoras de economía circular en el departamento.</t>
+        </is>
+      </c>
+      <c r="U306" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: reconoce iniciativas en economía circular territorial, posible alineación con modelos de negocio circulares, inclusión de actores regionales y sostenibilidad empresarial.</t>
+        </is>
+      </c>
+      <c r="V306" t="inlineStr">
+        <is>
+          <t>Iniciativas de cierre de ciclo regional (Cauca); Modelos de negocio circular territoriales; Reciclaje y aprovechamiento de residuos; Ecodiseño; Inclusión de recicladores informales.</t>
+        </is>
+      </c>
+      <c r="W306" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X306" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y306" t="inlineStr">
+        <is>
+          <t>Autoridades departamentales del Cauca; Recicladores organizados de la región; Empresas locales de gestión ambiental; Universidades del Cauca; Gremios regionales.</t>
+        </is>
+      </c>
+      <c r="Z306" t="inlineStr">
+        <is>
+          <t>CONVOCATORIA CERRANDO HOY. Ventana de postulación extremadamente reducida (solo horas restantes). Sin bases detalladas en fuentes accesibles. Requiere acción inmediata si hay iniciativas preparadas.</t>
+        </is>
+      </c>
+      <c r="AA306" t="inlineStr">
+        <is>
+          <t>URGENTE: Contactar inmediatamente a Urbaser (https://urbaser.co/premio-economia-circular) para obtener bases y formulario. Si hay iniciativa preparada de Visión Circular en Cauca, postular HOY. Si no, documentar para próxima edición 2027.</t>
+        </is>
+      </c>
+      <c r="AB306" t="inlineStr">
+        <is>
+          <t>1) AHORA: Acceder a https://urbaser.co/premio-economia-circular; 2) Descargar bases y formulario; 3) Si existe iniciativa elegible, completar y enviar antes de fin de día (2026-04-08); 4) Si no, recopilar lecciones y preparar para 2027.</t>
+        </is>
+      </c>
+      <c r="AC306" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos (acción inmediata); Alianzas regionales Cauca.</t>
+        </is>
+      </c>
+      <c r="AD306" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE306" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF306" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG306" t="inlineStr">
+        <is>
+          <t>Fuente confiable (Facebook oficial Urbaser Popayán). Premio activo y vigente. CRÍTICO: Cierre HOY. Elegibilidad depende de cobertura geográfica (¿solo Cauca o regional?) y tipo de soluciones aceptadas (iniciativas, empresas, recicladores). Requiere verificación urgente de bases. | Fuente fuera del listado oficial conocido (urbaser.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH306" t="inlineStr">
+        <is>
+          <t>4a3b0bac8b3204ea</t>
+        </is>
+      </c>
+      <c r="AI306" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>VC-0306</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Proyecto MarColombia - Cooperación Países Bajos</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Gobierno de los Países Bajos (Embajada de los Países Bajos en Colombia)</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Países Bajos</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Residuos y reciclaje</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Gestión de residuos sólidos; cadena de reciclaje; herramientas tecnológicas para trazabilidad; política de residuos</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Investigación aplicada; Innovación</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>Proyecto activo (iniciado hace ~3 años, estado actual desconocido)</t>
+        </is>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>https://www.minvivienda.gov.co/ministerio/gestion-institucional/cooperacion-internacional</t>
+        </is>
+      </c>
+      <c r="S307" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T307" t="inlineStr">
+        <is>
+          <t>Proyecto de cooperación bilateral Países Bajos-Colombia enfocado en fortalecer la política de gestión de residuos sólidos. Ha desarrollado y pilotado una herramienta tecnológica para recopilar información de la cadena de reciclaje con participación de actores del sector. Estado actual: requiere verificación sobre fase vigente y oportunidades de ampliación.</t>
+        </is>
+      </c>
+      <c r="U307" t="inlineStr">
+        <is>
+          <t>Muy pertinente: directamente relacionado con gestión de residuos, trazabilidad de cadena de reciclaje e innovación tecnológica. Alineado con objetivos de Visión Circular en cierre de ciclos, inclusión y articulación.</t>
+        </is>
+      </c>
+      <c r="V307" t="inlineStr">
+        <is>
+          <t>Fortalecimiento de herramienta tecnológica de trazabilidad de reciclaje; escalamiento de solución digital a nivel nacional; inclusión de recicladores en cadena de información; piloto demostrativo en nuevas regiones; capacitación en uso de plataforma; validación de política de gestión de residuos.</t>
+        </is>
+      </c>
+      <c r="W307" t="inlineStr">
+        <is>
+          <t>Ser entidad pública colombiana (Ministerio de Vivienda u organismos sectores afines); participación de actores de cadena de reciclaje; capacidad de implementación local; alianzas con municipios, recicladores u organizaciones del sector.</t>
+        </is>
+      </c>
+      <c r="X307" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto; presupuesto; plan de implementación; cartas de respaldo institucional; estudios de viabilidad; documentación de actores participantes; No especificado.</t>
+        </is>
+      </c>
+      <c r="Y307" t="inlineStr">
+        <is>
+          <t>Ministerio de Vivienda, Ciudad y Territorio; Embajada de los Países Bajos; municipalidades; autoridades ambientales; gremios de recicladores; empresas de residuos; centros tecnológicos.</t>
+        </is>
+      </c>
+      <c r="Z307" t="inlineStr">
+        <is>
+          <t>Información limitada y desactualizada (fuente menciona que proyecto 'nació hace casi tres años'); desconocimiento de fase actual (¿activo?, ¿en evaluación?, ¿cierre?); posible falta de presupuesto disponible; requiere verificación con MVCT sobre continuidad y amplificación.</t>
+        </is>
+      </c>
+      <c r="AA307" t="inlineStr">
+        <is>
+          <t>Contactar directamente Ministerio de Vivienda (MVCT) y Embajada de los Países Bajos para: 1) obtener estado actual del proyecto MarColombia; 2) identificar si hay convocatoria abierta para nuevas alianzas; 3) evaluación de oportunidad de ANDI como socio implementador o de articulación.</t>
+        </is>
+      </c>
+      <c r="AB307" t="inlineStr">
+        <is>
+          <t>1. Solicitar información oficial a MVCT sobre estado de MarColombia y oportunidades de participación; 2. Contactar Embajada de Países Bajos (cooperación técnica); 3. Revisar herramienta tecnológica existente para entender su aplicabilidad a Visión Circular; 4. Evaluar alianza con recicladores y municipios.</t>
+        </is>
+      </c>
+      <c r="AC307" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos; Especialista en Tecnología y Trazabilidad; Coordinación de Alianzas con Gobierno.</t>
+        </is>
+      </c>
+      <c r="AD307" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE307" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF307" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG307" t="inlineStr">
+        <is>
+          <t>Fuente: sitio oficial de Minvivienda. La información es limitada (solo 2 párrafos contextuales); no hay fecha de cierre ni detalles de convocatoria visible. Inferencia: proyecto aparentemente activo pero requiere verificación sobre si aún acepta nuevos aliados o si está en fase de cierre/evaluación. El componente de herramienta tecnológica es muy alineado con Visión Circular. | Fuente fuera del listado oficial conocido (minvivienda.gov.co): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH307" t="inlineStr">
+        <is>
+          <t>7f1c8483b1e419c9</t>
+        </is>
+      </c>
+      <c r="AI307" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>VC-0307</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Convocatoria Social de Cooperación Internacional 2026 - La Caixa</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Fundación La Caixa</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Fundación</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Mozambique, Perú, Colombia</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Innovación social; sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>Iniciativas de innovación social (potencial aplicación a economía circular, gestión de residuos, inclusión de recicladores)</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Innovación</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>https://fundacionlacaixa.org/es/cooperacion-internacional-convocatoria</t>
+        </is>
+      </c>
+      <c r="S308" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T308" t="inlineStr">
+        <is>
+          <t>Convocatoria abierta de La Caixa para innovación social en Colombia, Perú y Mozambique. Ventana de candidaturas: 15 de abril a 20 de mayo de 2026. Financia proyectos de innovación social con impacto territorial y comunitario.</t>
+        </is>
+      </c>
+      <c r="U308" t="inlineStr">
+        <is>
+          <t>Relevancia media-alta: convocatoria de innovación social abierta a Colombia permite postular iniciativas de economía circular con impacto social (ej. inclusión de recicladores, modelos de negocio circulares inclusivos, ecodiseño comunitario).</t>
+        </is>
+      </c>
+      <c r="V308" t="inlineStr">
+        <is>
+          <t>Modelos de negocio circular inclusivos; fortalecimiento de cooperativas de recicladores; plataformas de innovación en economía circular; ecodiseño participativo; iniciativas de cierre de ciclos con componente de inclusión social.</t>
+        </is>
+      </c>
+      <c r="W308" t="inlineStr">
+        <is>
+          <t>Ser organización (ONG, empresa social, gremio, consorcio) con capacidad de implementación en Colombia; demostrar impacto social; presentar proyecto de innovación; No especificado (requiere acceso a bases).</t>
+        </is>
+      </c>
+      <c r="X308" t="inlineStr">
+        <is>
+          <t>Formulario de candidatura de La Caixa; descripción de proyecto; presupuesto; plan de impacto social; documentos legales de organización; cartas de apoyo; No especificado.</t>
+        </is>
+      </c>
+      <c r="Y308" t="inlineStr">
+        <is>
+          <t>ONG ambientales; cooperativas de recicladores; municipalidades; gremios (ANDI); empresas privadas; universidades; centros tecnológicos.</t>
+        </is>
+      </c>
+      <c r="Z308" t="inlineStr">
+        <is>
+          <t>Ventana muy corta (35 días entre apertura y cierre); convocatoria ya cerrada (fecha límite 20 de mayo de 2026, que es en pasado respecto a búsqueda de 'hoy'); no hay garantía de que tema sea economía circular explícito (es 'innovación social' genérica); montos desconocidos.</t>
+        </is>
+      </c>
+      <c r="AA308" t="inlineStr">
+        <is>
+          <t>Verificar si convocatoria 2026 de La Caixa ya cerró o si hay nueva edición 2027 abierta. Si la convocatoria citada (abril-mayo 2026) ya cerró, contactar La Caixa para calendarios futuros. De estar abierta aún, preparar proyecto piloto de innovación circular con inclusión social para Colombia.</t>
+        </is>
+      </c>
+      <c r="AB308" t="inlineStr">
+        <is>
+          <t>1. Verificar estado de convocatoria La Caixa 2026 (verificar si hoy es antes o después del 20 mayo 2026); 2. Si cerrada, registrarse en plataforma de La Caixa para convocatorias futuras; 3. Si abierta aún, preparar propuesta de innovación circular con foco social.</t>
+        </is>
+      </c>
+      <c r="AC308" t="inlineStr">
+        <is>
+          <t>Coordinación de Innovación y Proyectos Especiales; Especialista en Inclusión Social.</t>
+        </is>
+      </c>
+      <c r="AD308" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE308" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF308" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG308" t="inlineStr">
+        <is>
+          <t>Fuente: sitio oficial de La Caixa. La convocatoria es específica de 2026 con ventana abril-mayo. Contextualmente, si la búsqueda es de 'hoy' (momento actual desconocido), la convocatoria puede ya estar cerrada. Es una oportunidad válida pero requiere urgente verificación de vigencia. No está explícitamente orientada a economía circular, pero 'innovación social' en residuos/reciclaje sería aplicable. | Fuente fuera del listado oficial conocido (fundacionlacaixa.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH308" t="inlineStr">
+        <is>
+          <t>0373f00b4198d866</t>
+        </is>
+      </c>
+      <c r="AI308" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>VC-0308</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Convocatoria Regional de Soluciones Innovadoras en Plásticos - Cempre Colombia, WRAP y Red Global de Pactos por los Plásticos</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Cempre Colombia; WRAP (organización internacional de acción climática); Red Global de Pactos por los Plásticos</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral; ONG</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Internacional (WRAP con presencia global)</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Colombia, México, Chile</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Economía circular; Envases y empaques; Plásticos</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>Soluciones empresariales innovadoras para gestión sostenible de envases y empaques plásticos</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Financiamiento concesional; Innovación</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>Hasta USD 10.000 por solución</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>2025-11 (Abierta)</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>https://www.pactoglobal-colombia.org/news/convocatoria-regional-otorgara-hasta-usd-10-000-a-soluciones-innovadoras-en-plasticos-en-colombia-chile-y-mexico.html</t>
+        </is>
+      </c>
+      <c r="S309" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T309" t="inlineStr">
+        <is>
+          <t>Convocatoria regional abierta que identifica e impulsa 10 soluciones empresariales innovadoras para la gestión sostenible de envases y empaques plásticos. Financia hasta USD 10.000 por solución en Colombia, México y Chile. Liderada por Cempre Colombia, WRAP y Red Global de Pactos por los Plásticos.</t>
+        </is>
+      </c>
+      <c r="U309" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: aborda directamente innovación en envases/empaques, modelos de negocio circulares y sostenibilidad de plásticos, ejes centrales de Visión Circular ANDI.</t>
+        </is>
+      </c>
+      <c r="V309" t="inlineStr">
+        <is>
+          <t>Innovación en ecodiseño de envases; Modelos de negocio circulares para empaques plásticos; Soluciones de reciclabilidad; Reducción de plásticos de un solo uso; Pilotos empresariales de economía circular</t>
+        </is>
+      </c>
+      <c r="W309" t="inlineStr">
+        <is>
+          <t>No especificado (requiere verificación en fuente oficial)</t>
+        </is>
+      </c>
+      <c r="X309" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y309" t="inlineStr">
+        <is>
+          <t>Cempre Colombia (como socio local); WRAP; Empresas empaques ANDI; Universidades y centros tecnológicos; Organizaciones de recicladores</t>
+        </is>
+      </c>
+      <c r="Z309" t="inlineStr">
+        <is>
+          <t>Monto por solución es acotado (USD 10.000); no se especifican requisitos ni cronograma de cierre; requiere confirmación de elegibilidad de actores no empresariales (gremios, ONG, universidades)</t>
+        </is>
+      </c>
+      <c r="AA309" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a Cempre Colombia para obtener bases de la convocatoria y verificar elegibilidad de ANDI como entidad articuladora de empresas. Preparar portafolio de 2-3 soluciones innovadoras de empresas afiliadas.</t>
+        </is>
+      </c>
+      <c r="AB309" t="inlineStr">
+        <is>
+          <t>1) Verificar en Cempre Colombia términos exactos y fecha cierre; 2) Revisar si ANDI puede presentar como articulador o si deben hacerlo empresas directamente; 3) Socializar con empresas miembro ANDI; 4) Preparar fichas técnicas de innovaciones candidatas</t>
+        </is>
+      </c>
+      <c r="AC309" t="inlineStr">
+        <is>
+          <t>Coordinación de Innovación / Alianzas Empresariales; contacto con Cempre Colombia</t>
+        </is>
+      </c>
+      <c r="AD309" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE309" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF309" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG309" t="inlineStr">
+        <is>
+          <t>Convocatoria confirmada en noviembre 2025 (actual). Instagram del 4 de diciembre 2025 indica 'Ya está abierta'. No hay URL directa de bases ni fecha cierre explícita en la fuente. Muy reciente y altamente compatible con Visión Circular. Requiere verificación de detalles operativos. | Fuente fuera del listado oficial conocido (pactoglobal-colombia.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH309" t="inlineStr">
+        <is>
+          <t>82d406035c1d1557</t>
+        </is>
+      </c>
+      <c r="AI309" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>VC-0309</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>CircularEconomy4Colombia: Agrichallenge</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>No especificado (inferred: Agritech Alliance o consorcio internacional)</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>Colombia (foco específico)</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>Transición a economía circular en sector agrícola y agroindustrial</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Aceleración; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P310" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R310" t="inlineStr">
+        <is>
+          <t>https://agritechchallenge.org/projects/circulareconomy-4colombia</t>
+        </is>
+      </c>
+      <c r="S310" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T310" t="inlineStr">
+        <is>
+          <t>Challenge innovador alineado con el Plan Nacional de Desarrollo 2022-2026 de Colombia y objetivos de la COP 16 CBD. Ofrece mentorización experta y apoyo integral para acelerar soluciones de economía circular en el sector agrícola y agroindustrial colombiano, con potencial de impacto en cadenas de valor y sostenibilidad.</t>
+        </is>
+      </c>
+      <c r="U310" t="inlineStr">
+        <is>
+          <t>Altamente relevante: aborda economía circular territorial, cierre de ciclo de materiales, modelos de negocio circulares y articulación con empresas gremiales en sector estratégico. Alineado directamente con ENEC (Estrategia Nacional de Economía Circular de Colombia).</t>
+        </is>
+      </c>
+      <c r="V310" t="inlineStr">
+        <is>
+          <t>Pilotos empresariales en agroindustria; Modelos de negocio circulares para cadenas agroalimentarias; Ecodiseño de envases y empaques agrícolas; Inclusión de recicladores en cadenas de valor agroindustriales; Cierre de ciclo de residuos agroindustriales</t>
+        </is>
+      </c>
+      <c r="W310" t="inlineStr">
+        <is>
+          <t>No especificado (típicamente: solución innovadora de economía circular, aplicable en Colombia, fase de prototipo o validación, equipo con capacidad de ejecución)</t>
+        </is>
+      </c>
+      <c r="X310" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y310" t="inlineStr">
+        <is>
+          <t>Gremios agrícolas (Fedegan, Asocaña, Asohofrucol), universidades agrícolas (Universidad Nacional, Javeriana), asociaciones de recicladores, empresas de procesamiento agroindustrial</t>
+        </is>
+      </c>
+      <c r="Z310" t="inlineStr">
+        <is>
+          <t>No especificado; posible sesgo hacia startups/innovadores vs. actores tradicionales de reciclaje</t>
+        </is>
+      </c>
+      <c r="AA310" t="inlineStr">
+        <is>
+          <t>Contactar directamente con organización coordinadora para validar: (1) fechas de convocatoria 2025, (2) monto de premios/apoyo, (3) eligibilidad de ANDI como articuladora vs. solo soluciones innovadoras individuales, (4) oportunidades de alianza con gremios afiliados.</t>
+        </is>
+      </c>
+      <c r="AB310" t="inlineStr">
+        <is>
+          <t>Revisar sitio https://agritechchallenge.org completo; contactar coordinadores del challenge; explorar si ANDI puede participar como facilitador de empresas miembro; preparar mapeo de 2-3 casos piloto en agroindustria alineados con Visión Circular.</t>
+        </is>
+      </c>
+      <c r="AC310" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos y alianzas; Especialista en agricultura sostenible/agroindustria</t>
+        </is>
+      </c>
+      <c r="AD310" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE310" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF310" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG310" t="inlineStr">
+        <is>
+          <t>Challenge existente y activo, pero sin fechas exactas de cierre ni monto disponible en fuente. Inferencia: abierto permanentemente o con convocatorias periódicas. Altamente alineado con mandato de Visión Circular en pilotos y modelos de negocio. Requiere verificación de vigencia y plazos actuales. | Fuente fuera del listado oficial conocido (agritechchallenge.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH310" t="inlineStr">
+        <is>
+          <t>5e6ab6b8ead01b43</t>
+        </is>
+      </c>
+      <c r="AI310" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>VC-0310</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Circulate Capital - Apply for Funding (Recycling Supply Chains)</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Circulate Capital</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Fondo | Fundación</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>América Latina (incluida Colombia)</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Reciclaje</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>Cadenas de suministro de reciclaje, recolección y clasificación, tecnologías de upcycling, digitalización</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Innovación; Escalamiento</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N311" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente</t>
+        </is>
+      </c>
+      <c r="P311" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q311" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R311" t="inlineStr">
+        <is>
+          <t>https://www.circulatecapital.com/apply-for-funding</t>
+        </is>
+      </c>
+      <c r="S311" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T311" t="inlineStr">
+        <is>
+          <t>Circulate Capital financia iniciativas de economía circular en América Latina enfocadas en cadenas de reciclaje, recolección y clasificación de residuos, tecnologías de upcycling y digitalización de supply chains. La plataforma busca eliminar el escape de residuos al ambiente y mejorar la eficiencia y trazabilidad en procesos de reciclaje mediante tecnologías de big data e IA.</t>
+        </is>
+      </c>
+      <c r="U311" t="inlineStr">
+        <is>
+          <t>Altamente alineada: financia directamente cierre de ciclo de envases, cadenas de reciclaje, innovación en reciclabilidad y tecnologías para inclusión y eficiencia de recicladores formales e informales.</t>
+        </is>
+      </c>
+      <c r="V311" t="inlineStr">
+        <is>
+          <t>Pilotos empresariales de recolección y clasificación; Tecnologías de upcycling de plásticos flexibles; Plataformas digitales para trazabilidad de envases y empaques; Modelos de negocio inclusivos con recicladores; Sistemas de articulación empresa-reciclador.</t>
+        </is>
+      </c>
+      <c r="W311" t="inlineStr">
+        <is>
+          <t>No especificado (requiere verificación en sitio web)</t>
+        </is>
+      </c>
+      <c r="X311" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y311" t="inlineStr">
+        <is>
+          <t>Empresas de envases y empaques; gremios como ANDI; cooperativas de recicladores; startups de tecnología ambiental; centros tecnológicos de investigación en reciclaje.</t>
+        </is>
+      </c>
+      <c r="Z311" t="inlineStr">
+        <is>
+          <t>Fondo probablemente enfocado en proyectos con potencial de retorno financiero; puede haber requisitos de tasa de descuento o modelo de negocio rentable.</t>
+        </is>
+      </c>
+      <c r="AA311" t="inlineStr">
+        <is>
+          <t>Contactar directamente a Circulate Capital con propuestas de pilotos empresariales de recolección/clasificación de envases y tecnologías de upcycling de plásticos flexibles; preparar business case con proyecciones de impacto ambiental y retorno.</t>
+        </is>
+      </c>
+      <c r="AB311" t="inlineStr">
+        <is>
+          <t>1) Revisar sitio web completo para identificar criterios de elegibilidad y formulario; 2) Preparar documento de 2-3 págs con descripción del proyecto, modelo de negocio y presupuesto estimado; 3) Contactar a Circulate Capital vía sitio oficial.</t>
+        </is>
+      </c>
+      <c r="AC311" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos / Alianzas empresariales</t>
+        </is>
+      </c>
+      <c r="AD311" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE311" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF311" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG311" t="inlineStr">
+        <is>
+          <t>Circulate Capital opera activamente en América Latina. URL confirma operación en geografía LAC. Requiere verificación de montos, plazos específicos y criterios de elegibilidad detallados accediendo al formulario en línea.</t>
+        </is>
+      </c>
+      <c r="AH311" t="inlineStr">
+        <is>
+          <t>aef749565caf689c</t>
+        </is>
+      </c>
+      <c r="AI311" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>VC-0311</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Joint SDG Fund - Green Finance for Circular Economy in Colombia</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Joint SDG Fund (PNUD + gobiernos)</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral | Fondo climático</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Global (Naciones Unidas)</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>Financiamiento verde, modelos de negocio circular, reducción de residuos, eficiencia de recursos</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Financiamiento concesional; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N312" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P312" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q312" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R312" t="inlineStr">
+        <is>
+          <t>https://jointsdgfund.org/article/colombia-unlocks-green-finance-more-circular-economy</t>
+        </is>
+      </c>
+      <c r="S312" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T312" t="inlineStr">
+        <is>
+          <t>Iniciativa de Naciones Unidas (Joint SDG Fund) que conecta las ambiciones de economía circular de Colombia con financiamiento verde. El programa trabaja para cerrar la brecha entre empresas colombianas que desean adoptar modelos de negocio circular y el acceso a financiamiento adecuado para reducir residuos y usar recursos de manera eficiente.</t>
+        </is>
+      </c>
+      <c r="U312" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: alinea directamente políticas de economía circular de Colombia con instrumentos financieros; facilita adopción de modelos de negocio circulares en empresas y articulación con finanzas verdes.</t>
+        </is>
+      </c>
+      <c r="V312" t="inlineStr">
+        <is>
+          <t>Financiamiento para pilotos de economía circular en empresas; Acceso a financiamiento verde para transición a producción más sostenible; Fortalecimiento de marcos de política pública para economía circular; Articulación empresa-gobierno para implementación de REP.</t>
+        </is>
+      </c>
+      <c r="W312" t="inlineStr">
+        <is>
+          <t>No especificado (programa general de articulación)</t>
+        </is>
+      </c>
+      <c r="X312" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y312" t="inlineStr">
+        <is>
+          <t>PNUD Colombia; Ministerio de Ambiente y Desarrollo Sostenible; ANDI como gremio empresarial; bancos e instituciones financieras colombianas; empresas interesadas en modelos circulares.</t>
+        </is>
+      </c>
+      <c r="Z312" t="inlineStr">
+        <is>
+          <t>Nivel de detalle muy general en fuente; requiere contacto directo con Joint SDG Fund / PNUD para acceder a convocatorias específicas.</t>
+        </is>
+      </c>
+      <c r="AA312" t="inlineStr">
+        <is>
+          <t>Contactar a PNUD Colombia y Joint SDG Fund para identificar convocatorias activas; posicionar a ANDI / Visión Circular como aliado estratégico en articulación empresa-gobierno-finanzas.</t>
+        </is>
+      </c>
+      <c r="AB312" t="inlineStr">
+        <is>
+          <t>1) Contactar PNUD Colombia (oficina de Economía Circular o SDG Finance); 2) Solicitar información sobre convocatorias vigentes y criterios de elegibilidad; 3) Evaluar si Visión Circular puede actuar como facilitador de alianzas empresa-financiamiento.</t>
+        </is>
+      </c>
+      <c r="AC312" t="inlineStr">
+        <is>
+          <t>Alianzas estratégicas / Coordinación interinstitucional</t>
+        </is>
+      </c>
+      <c r="AD312" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE312" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF312" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG312" t="inlineStr">
+        <is>
+          <t>Fuente es artículo de Joint SDG Fund (entidad oficial de la ONU). No hay fechas, montos ni formularios específicos en la búsqueda. Es probable que existan convocatorias y líneas operativas activas vía PNUD Colombia, pero requieren verificación directa. | Fuente fuera del listado oficial conocido (jointsdgfund.org): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH312" t="inlineStr">
+        <is>
+          <t>8d71cc2d9de218f5</t>
+        </is>
+      </c>
+      <c r="AI312" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>VC-0312</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Colombia's Green Jobs Programme - Supporting Colombia's Transition to a Circular Economy</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>GOPA (Gesellschaft für Organisation, Planung und Ausbildung mbH)</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Sistemas de reciclaje inclusivo, empleo verde, políticas de economía circular, acción climática territorial</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Asistencia técnica; Fortalecimiento institucional; Inclusión social</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N313" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P313" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R313" t="inlineStr">
+        <is>
+          <t>https://www.gopa.eu/en/projects/flagship/colombia-green-jobs-circular-economy</t>
+        </is>
+      </c>
+      <c r="S313" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T313" t="inlineStr">
+        <is>
+          <t>Programa de cooperación bilateral GOPA enfocado en ayudar a ciudades colombianas a convertir políticas de economía circular en sistemas de reciclaje mejorados, empleo inclusivo y acción climática local. Ofrece asistencia técnica y fortalecimiento institucional para la transición circular en Colombia.</t>
+        </is>
+      </c>
+      <c r="U313" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: aborda directamente sistemas de reciclaje, inclusión laboral de recicladores, políticas de economía circular e implementación territorial, pilares estratégicos de Visión Circular ANDI.</t>
+        </is>
+      </c>
+      <c r="V313" t="inlineStr">
+        <is>
+          <t>Pilotos empresariales de reciclaje inclusivo; Articulación con autoridades locales para políticas de economía circular; Modelos de negocio circulares en ciudades; Inclusión de recicladores en cadenas formales; Fortalecimiento de capacidades en gremios y municipios.</t>
+        </is>
+      </c>
+      <c r="W313" t="inlineStr">
+        <is>
+          <t>Ser entidad pública, gremio, empresa o alianza en Colombia con interés en transición circular; Capacidad de implementación territorial; Disposición para co-crear con GOPA.</t>
+        </is>
+      </c>
+      <c r="X313" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y313" t="inlineStr">
+        <is>
+          <t>ANDI como gremio coordinador; Municipios y ciudades colombianas; Autoridades ambientales; Universidades y centros tecnológicos; Organizaciones de recicladores; Empresas del sector de envases/empaques.</t>
+        </is>
+      </c>
+      <c r="Z313" t="inlineStr">
+        <is>
+          <t>Información limitada sobre vigencia exacta y proceso de aplicación; requiere contacto directo con GOPA para validar disponibilidad de recursos y cronograma.</t>
+        </is>
+      </c>
+      <c r="AA313" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a GOPA para validar si el programa sigue activo, presupuesto disponible y ventanas de aplicación; Posicionar a ANDI como coordinador estratégico de alianzas colombianas.</t>
+        </is>
+      </c>
+      <c r="AB313" t="inlineStr">
+        <is>
+          <t>1) Enviar correo de interés a GOPA con propuesta conceptual de colaboración; 2) Identificar 2-3 ciudades/gremios piloto en Colombia; 3) Preparar carta de intención conjunta ANDI-municipios.</t>
+        </is>
+      </c>
+      <c r="AC313" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos / Alianzas Estratégicas</t>
+        </is>
+      </c>
+      <c r="AD313" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE313" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF313" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG313" t="inlineStr">
+        <is>
+          <t>Proyecto flagshipde GOPA explícitamente diseñado para Colombia. Información disponible sugiere vigencia activa, pero no hay detalles sobre convocatorias abiertas, montos o fechas. Requiere verificación de estado operativo. | Fuente fuera del listado oficial conocido (gopa.eu): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH313" t="inlineStr">
+        <is>
+          <t>c22f2b4bac9c4248</t>
+        </is>
+      </c>
+      <c r="AI313" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>VC-0313</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Horizon Europe: Circular Economy – Advanced Materials for Circularity</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>European Commission (Comisión Europea) / Horizon Europe Programme</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral (Unión Europea)</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Estados miembros UE, países asociados Horizon Europe (requiere verificación si incluye LATAM o alianzas)</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>Materiales avanzados reciclables, polímeros reciclables, bioplásticos, composite circulares, manufactura aditiva</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Investigación aplicada; Innovación</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>No especificado (típicamente Horizon Europe: EUR 500k-5M+)</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>No especificado; típicamente en Horizon Europe: cofinanciación variable (algunos llaman R&amp;I: 100%, algunos requieren 20-30%)</t>
+        </is>
+      </c>
+      <c r="N314" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>2026-09-24 (estimado como deadline de call)</t>
+        </is>
+      </c>
+      <c r="P314" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q314" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R314" t="inlineStr">
+        <is>
+          <t>https://eufundingportal.eu/circular-economy</t>
+        </is>
+      </c>
+      <c r="S314" t="inlineStr">
+        <is>
+          <t>ec.europa.eu/research/participants/portal (inferida)</t>
+        </is>
+      </c>
+      <c r="T314" t="inlineStr">
+        <is>
+          <t>Horizon Europe financia innovación en materiales avanzados diseñados para circularidad (polímeros reciclables, composites, aleaciones, magnetos) aplicables a manufactura aditiva y cadenas circulares. Call abierto hasta septiembre 2026. Acceso típicamente para consorcios de investigación/industria UE + aliados.</t>
+        </is>
+      </c>
+      <c r="U314" t="inlineStr">
+        <is>
+          <t>Muy relevante: cubre ecodiseño, reciclabilidad de materiales, innovación en empaques reciclables y polímeros avanzados; alineado con línea de reciclaje y materiales circulares de Visión Circular.</t>
+        </is>
+      </c>
+      <c r="V314" t="inlineStr">
+        <is>
+          <t>Investigación aplicada en polímeros reciclables y composites para envases; Ecodiseño de empaques avanzados; Innovación en bioplásticos y biocomposites circulares; Pilotos de manufactura aditiva con materiales reciclables; Transferencia de tecnología a PYMES europeas y aliados.</t>
+        </is>
+      </c>
+      <c r="W314" t="inlineStr">
+        <is>
+          <t>Consorcio multinacional mínimo (típicamente 3+ socios); al menos 50% de participantes de Estados Miembros/Asociados UE. LATAM puede participar como socio de bajo costo (típicamente 25% máximo de budget) o en co-financiación. Capacidad técnica y financiera requeridas.</t>
+        </is>
+      </c>
+      <c r="X314" t="inlineStr">
+        <is>
+          <t>Propuesta técnica (max 15 páginas), trabajo plan, presupuesto detallado, CV de coordinadores, letter of commitment de socios, datos de capacidad financiera/técnica de cada institución.</t>
+        </is>
+      </c>
+      <c r="Y314" t="inlineStr">
+        <is>
+          <t>Universidades/centros de investigación UE (especialistas en polímeros, materials science); empresas plásticas europeas (Tupperware, Huhtamaki, etc.); centros tecnológicos LATAM (INTI Argentina, SENAI Brasil, SENA Colombia) como socios; gremios ANDI via ACOPLÁSTICOS.</t>
+        </is>
+      </c>
+      <c r="Z314" t="inlineStr">
+        <is>
+          <t>Elegibilidad LATAM limitada a rol de socio de bajo costo; requiere consorcio líder UE. Competencia muy alta (Horizon Europe: tasa de éxito ~13%). Complejidad administrativa elevada. Ventana de 2026 sugiere deadline lejano.</t>
+        </is>
+      </c>
+      <c r="AA314" t="inlineStr">
+        <is>
+          <t>Posibilidad MEDIA: ANDI/Visión Circular puede actuar como socio de investigación aplicada + transferencia (bajo costo) en propuesta liderada por institución UE. Recomendar identificar partner europeo interesado en cadenas circulares LATAM (packaging, reciclaje, inclusión social).</t>
+        </is>
+      </c>
+      <c r="AB314" t="inlineStr">
+        <is>
+          <t>1) Monitorear próximas aperturas Horizon Europe 2026 en ec.europa.eu/research; 2) Mapear universidades/centros UE con expertise en polímeros + interés LATAM (ej. ICLG Italia, Fraunhofer Alemania); 3) Evaluar capacidad de ANDI para participar como socio de investigación aplicada (sin ser coordinador).</t>
+        </is>
+      </c>
+      <c r="AC314" t="inlineStr">
+        <is>
+          <t>Coordinación de alianzas internacionales; Área de investigación e innovación; Cooperación UE.</t>
+        </is>
+      </c>
+      <c r="AD314" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE314" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF314" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG314" t="inlineStr">
+        <is>
+          <t>Información de eufundingportal.eu (fuente confiable pero secundaria). Deadline 2026-09-24 es estimación del portal. Montos típicos de Horizon Europe: €500k-€5M, pero no confirmados para este call. LATAM elegibilidad: parcial como socio en consorcio, no como coordinador. Requiere verificación en European Commission portal oficial. | Fuente fuera del listado oficial conocido (eufundingportal.eu): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH314" t="inlineStr">
+        <is>
+          <t>1fc724b19222dba1</t>
+        </is>
+      </c>
+      <c r="AI314" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>VC-0314</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Inclusive Recycling: Government, Businesses, and Waste Pickers</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Banco Interamericano de Desarrollo (BID)</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Estados Unidos (sede regional para América Latina)</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (énfasis en países miembros del BID)</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Reciclaje, Residuos, Inclusión social</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>Inclusión de recicladores informales, Responsabilidad Extendida del Productor (REP), Formalización de sistemas de reciclaje</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Piloto demostrativo; Fortalecimiento institucional; Inclusión social</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N315" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P315" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q315" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R315" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/project/CH-M1055</t>
+        </is>
+      </c>
+      <c r="S315" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T315" t="inlineStr">
+        <is>
+          <t>El BID desarrolla un proyecto para formalizar sistemas de reciclaje inclusivo vinculados a la Responsabilidad Extendida del Productor (REP). El modelo busca ser sostenible y replicable en diferentes territorios del país, articulando empresas, municipios, recicladores y comunidades en una cadena integrada de valor.</t>
+        </is>
+      </c>
+      <c r="U315" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: aborda directamente REP, inclusión de recicladores informales, formalización de sistemas de reciclaje y modelos de negocio circular territorial, tres pilares centrales de Visión Circular ANDI.</t>
+        </is>
+      </c>
+      <c r="V315" t="inlineStr">
+        <is>
+          <t>Formalización de recicladores; Diseño e implementación de REP territorial; Modelos de negocio circulares con inclusión; Articulación público-privada en reciclaje; Piloto empresarial de circularidad.</t>
+        </is>
+      </c>
+      <c r="W315" t="inlineStr">
+        <is>
+          <t>Ser país miembro del BID; Instituciones públicas, empresas gremiales o consorcios empresariales como ejecutores; Voluntad de implementar REP; Capacidad de cofinanciación local o institucional.</t>
+        </is>
+      </c>
+      <c r="X315" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y315" t="inlineStr">
+        <is>
+          <t>ANDI como gremio coordinador; Municipios participantes; Asociaciones de recicladores; Empresas productoras de envases/empaques; Universidades para investigación aplicada; Autoridades ambientales (MADS, ANLA).</t>
+        </is>
+      </c>
+      <c r="Z315" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="AA315" t="inlineStr">
+        <is>
+          <t>Contactar directamente al BID para obtener detalles de vigencia, montos, calendario y elegibilidad de ANDI como coordinador. Verificar si hay convocatoria abierta para nueva fase o si existe documento de proyecto vigente.</t>
+        </is>
+      </c>
+      <c r="AB315" t="inlineStr">
+        <is>
+          <t>1) Acceder a https://www.iadb.org/en/project/CH-M1055 y descargar Project Information; 2) Contactar equipo BID (correo de proyecto manager si aparece); 3) Evaluar si es proyecto en ejecución actual o propuesta nueva.</t>
+        </is>
+      </c>
+      <c r="AC315" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos + Alianzas Estratégicas (Visión Circular)</t>
+        </is>
+      </c>
+      <c r="AD315" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE315" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF315" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG315" t="inlineStr">
+        <is>
+          <t>La URL oficial del BID parece ser una ficha de proyecto existente o finalizado en Chile. Se infiere que el modelo y metodología podrían ser replicables a Colombia. Requiere verificación de vigencia, estado actual del proyecto y oportunidades de replicación o nueva fase.</t>
+        </is>
+      </c>
+      <c r="AH315" t="inlineStr">
+        <is>
+          <t>0541fda999a6db29</t>
+        </is>
+      </c>
+      <c r="AI315" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>VC-0315</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>IDB Lab BlueTech for Waste Challenge - Resultados y continuidad</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>IDB Lab (Laboratorio de Innovación del Banco Interamericano de Desarrollo)</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Banca multilateral; Fondo de innovación</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>EE.UU. (sede en Washington); opera en América Latina y Caribe</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>América Latina y Caribe (ALC), incluyendo Colombia</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Economía circular; Residuos; Sostenibilidad ambiental</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>Reciclaje de plásticos, Residuos, Innovación en gestión de residuos, Inclusión social</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>Premio o challenge; Financiamiento concesional; Aceleración; Innovación</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>No especificado en búsqueda; requiere verificación de convocatoria específica</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>Típicamente sí en programas IDB Lab; requiere verificación</t>
+        </is>
+      </c>
+      <c r="N316" t="inlineStr">
+        <is>
+          <t>No especificado; convocatoria 2024 cerrada (resultados publicados recientemente)</t>
+        </is>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>Convocatoria anterior cerrada; próxima ventana no especificada</t>
+        </is>
+      </c>
+      <c r="P316" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q316" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R316" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/news/idb-lab-announces-results-bluetech-waste-challenge</t>
+        </is>
+      </c>
+      <c r="S316" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org (sitio principal IDB Lab para próximas convocatorias)</t>
+        </is>
+      </c>
+      <c r="T316" t="inlineStr">
+        <is>
+          <t>IDB Lab anuncia resultados de desafío BlueTech for Waste que financió innovaciones en gestión de residuos y economía circular en ALC. Ganadores incluyen proyectos de reuso de baterías, soluciones en plásticos flexibles y biomasa. Demuestra apetito de IDB por financiar innovación circular en la región.</t>
+        </is>
+      </c>
+      <c r="U316" t="inlineStr">
+        <is>
+          <t>Altamente relevante: IDB Lab ha premiado soluciones de economía circular, plásticos y residuos en ALC. Proyecto ganador de NUVI (República Dominicana) en plásticos flexibles es directamente comparable a iniciativas de Visión Circular. Evidencia de viabilidad y demanda regional.</t>
+        </is>
+      </c>
+      <c r="V316" t="inlineStr">
+        <is>
+          <t>Pilotos empresariales de reciclaje; Innovación en plásticos flexibles; Modelos de negocio circular; Inclusión de recicladores; Escalamiento de soluciones circulares de startups.</t>
+        </is>
+      </c>
+      <c r="W316" t="inlineStr">
+        <is>
+          <t>Entidades innovadoras (startups, SMEs, cooperativas); alineación con ODS; demostración de impacto social/ambiental; capacidad de implementación en ALC</t>
+        </is>
+      </c>
+      <c r="X316" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto; plan de negocio; presupuesto; CV de equipo; cartas de apoyo de stakeholders; plan de sostenibilidad</t>
+        </is>
+      </c>
+      <c r="Y316" t="inlineStr">
+        <is>
+          <t>Startups e innovadores colombianos; Cooperativas de recicladores; Gremios ANDI, ACOPLÁSTICOS; Universidades con I+D en circularidad; Gobiernos locales; IFC (brazo de inversiones del BID)</t>
+        </is>
+      </c>
+      <c r="Z316" t="inlineStr">
+        <is>
+          <t>Convocatoria específica aparentemente cerrada (2024); próximas fechas no especificadas. Competencia regional alta. Requiere capacidad de cofinanciación.</t>
+        </is>
+      </c>
+      <c r="AA316" t="inlineStr">
+        <is>
+          <t>Identificar próximas convocatorias BlueTech o análogas de IDB Lab. Preparar cartera de proyectos innovadores Visión Circular (pilotos de reciclaje, plásticos flexibles, inclusión de recicladores) para futuros challenges. Explorar alianza con IDB Lab para co-diseño de convocatoria específica en REP/envases.</t>
+        </is>
+      </c>
+      <c r="AB316" t="inlineStr">
+        <is>
+          <t>1) Suscribirse a alertas de IDB Lab (https://www.iadb.org). 2) Contactar directamente IDB Lab sobre fecha de próxima convocatoria BlueTech o similar. 3) Documentar proyectos piloto Visión Circular con potencial de escalamiento para futura propuesta. 4) Explorar si IDB Lab ofrece asistencia técnica para preparación de propuestas.</t>
+        </is>
+      </c>
+      <c r="AC316" t="inlineStr">
+        <is>
+          <t>Coordinación de Innovación y Piloto; Alianzas con Banca Multilateral</t>
+        </is>
+      </c>
+      <c r="AD316" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE316" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF316" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG316" t="inlineStr">
+        <is>
+          <t>Búsqueda captura publicación de resultados (reciente), no convocatoria abierta. Sin embargo, evidencia clara de que IDB Lab financia soluciones circulares en ALC. Proyecto ganador NUVI (plásticos flexibles, RD) es muy similar a líneas Visión Circular. Probabilidad de futura convocatoria es alta. IDB Lab típicamente relanza challenges anualmente o bienalmente.</t>
+        </is>
+      </c>
+      <c r="AH316" t="inlineStr">
+        <is>
+          <t>5fcebf4fe3ede094</t>
+        </is>
+      </c>
+      <c r="AI316" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>VC-0316</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Caribbean Loans Call for Proposals</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>IDB Lab (Inter-American Development Bank)</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Estados Unidos (sede)</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>Región Caribeña principalmente; potencialmente América Latina (requiere verificación)</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Economía circular; Innovación; Sostenibilidad empresarial</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>Financiamiento para empresas innovadoras; Modelos de negocio circulares; Escalamiento empresarial</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>Financiamiento concesional; Aceleración; Innovación</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N317" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P317" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q317" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R317" t="inlineStr">
+        <is>
+          <t>https://bidlab.org/en/home/caribbean-loans-call-proposals</t>
+        </is>
+      </c>
+      <c r="S317" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T317" t="inlineStr">
+        <is>
+          <t>Convocatoria de IDB Lab que ofrece financiamiento en forma de préstamos para empresas innovadoras en América Latina y el Caribe. Busca impulsar innovación e impacto mediante deuda concesional.</t>
+        </is>
+      </c>
+      <c r="U317" t="inlineStr">
+        <is>
+          <t>Moderadamente relevante si se enfoca en empresas de economía circular, reciclaje o sostenibilidad. Requiere verificación de que acepte proyectos de circularidad explícitamente.</t>
+        </is>
+      </c>
+      <c r="V317" t="inlineStr">
+        <is>
+          <t>Escalamiento de empresas de reciclaje y gestión de residuos; Modelos de negocio circulares; Inclusión de recicladores formalizados; Emprendimientos en ecodiseño o reciclabilidad</t>
+        </is>
+      </c>
+      <c r="W317" t="inlineStr">
+        <is>
+          <t>Ser empresa innovadora con impacto; estar registrada en región elegible; demostrar viabilidad financiera</t>
+        </is>
+      </c>
+      <c r="X317" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y317" t="inlineStr">
+        <is>
+          <t>Empresas ANDI con iniciativas circulares; Cooperativas de recicladores; Centros tecnológicos; Incubadoras de emprendimiento ambiental</t>
+        </is>
+      </c>
+      <c r="Z317" t="inlineStr">
+        <is>
+          <t>Enfoque primario aparente en Caribe; Colombia podría no estar en prioridad geográfica. Requiere verificación.</t>
+        </is>
+      </c>
+      <c r="AA317" t="inlineStr">
+        <is>
+          <t>Verificar elegibilidad de Colombia y empresas colombianas en términos de referencia; si aplica, preparar propuesta de empresa/cooperativa de reciclaje con modelo financiero sólido</t>
+        </is>
+      </c>
+      <c r="AB317" t="inlineStr">
+        <is>
+          <t>Acceder a https://bidlab.org/en/home/caribbean-loans-call-proposals y descargar términos; confirmar si Colombia está dentro de cobertura</t>
+        </is>
+      </c>
+      <c r="AC317" t="inlineStr">
+        <is>
+          <t>Coordinación financiera; Alianzas con empresas y cooperativas</t>
+        </is>
+      </c>
+      <c r="AD317" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE317" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF317" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG317" t="inlineStr">
+        <is>
+          <t>La convocatoria existe pero no hay claridad sobre si Colombia está incluida (fuente menciona 'Latin America and the Caribbean' pero énfasis en Caribbean). Muy probable requiera alianza con empresa caribeña o verificar si ANDI puede actuar como intermediario.</t>
+        </is>
+      </c>
+      <c r="AH317" t="inlineStr">
+        <is>
+          <t>585ca1dd47f301e4</t>
+        </is>
+      </c>
+      <c r="AI317" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>VC-0317</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>IDB Lab - Circulate Capital Partnership for Ocean-Bound Plastics</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>IDB Lab (Inter-American Development Bank) en alianza con Circulate Capital</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Banca multilateral; Fondo de inversión</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe, con énfasis en Región Caribeña</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Economía circular; Plásticos; Residuos; Océanos</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>Plásticos flexibles; Gestión de residuos marinos; Inclusión de recicladores; Modelos de negocio circulares</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Inversión; Capacitación técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N318" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O318" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P318" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q318" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R318" t="inlineStr">
+        <is>
+          <t>https://www.iadb.org/en/news/idb-lab-partners-circulate-capital-combat-ocean-bound-plastics</t>
+        </is>
+      </c>
+      <c r="S318" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T318" t="inlineStr">
+        <is>
+          <t>Asociación entre IDB Lab y Circulate Capital que combina inversión en economía circular (enfocada en plásticos que llegan al océano) con programa de fortalecimiento de capacidades, especialmente en Caribe. Busca construir pipeline de inversión en innovación sostenible.</t>
+        </is>
+      </c>
+      <c r="U318" t="inlineStr">
+        <is>
+          <t>Altamente relevante: aborda circularidad en plásticos, inclusión de actores de reciclaje, cadenas de valor y sostenibilidad marina. Alinea con pilares de Visión Circular en plásticos flexibles e inclusión.</t>
+        </is>
+      </c>
+      <c r="V318" t="inlineStr">
+        <is>
+          <t>Pilotos empresariales de reciclaje de plásticos; Inclusión de recicladores en cadenas formales; Modelos de negocio circulares para empaques; Asistencia técnica a cooperativas; REP enfocado en plásticos</t>
+        </is>
+      </c>
+      <c r="W318" t="inlineStr">
+        <is>
+          <t>Ser empresa u organización en América Latina/Caribe; demostrar impacto potencial en prevención de plásticos marinos; viabilidad de modelo de negocio</t>
+        </is>
+      </c>
+      <c r="X318" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y318" t="inlineStr">
+        <is>
+          <t>Empresas de empaques plásticos; Cooperativas de recicladores; Autoridades costeras; ONGs ambientales; Gremios de manufactura; Universidades con investigación en plásticos</t>
+        </is>
+      </c>
+      <c r="Z318" t="inlineStr">
+        <is>
+          <t>Énfasis geográfico en Caribe podría priorizar islas; enfoque en plásticos marinos podría excluir proyectos de residuos terrestres; requiere validar apertura para inversión o si solo es asistencia técnica</t>
+        </is>
+      </c>
+      <c r="AA318" t="inlineStr">
+        <is>
+          <t>Contactar directamente a Circulate Capital y/o IDB Lab para conocer convocatoria abierta y términos; preparar propuesta sobre reciclaje de plásticos flexibles con componente de inclusión de recicladores</t>
+        </is>
+      </c>
+      <c r="AB318" t="inlineStr">
+        <is>
+          <t>Buscar 'Circulate Capital' en Google y acceder a su plataforma de inversión; consultar con IDB Lab sobre ventana de aplicación y cómo se articula con empresas colombianas</t>
+        </is>
+      </c>
+      <c r="AC318" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos; Alianzas con recicladores y empresas de empaques</t>
+        </is>
+      </c>
+      <c r="AD318" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE318" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF318" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG318" t="inlineStr">
+        <is>
+          <t>Se infiere que hay una convocatoria abierta basada en la noticia de IDB, pero no hay URL directa a términos de referencia ni fechas. El programa incluye capacitación técnica además de inversión, lo que aumenta probabilidad de elegibilidad para ANDI como facilitador.</t>
+        </is>
+      </c>
+      <c r="AH318" t="inlineStr">
+        <is>
+          <t>a4378aaa4024b180</t>
+        </is>
+      </c>
+      <c r="AI318" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>VC-0318</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Too Good to Waste - IDB Initiative</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Inter-American Development Bank (IDB)</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Banca multilateral</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Economía circular; Residuos; Sostenibilidad empresarial</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>Reutilización de materiales; Cadenas de valor circulares; Modelos de negocio circulares; Cierre de ciclo</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Aceleración; Innovación; Piloto demostrativo</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N319" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P319" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q319" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R319" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/BancoInteramericano/posts/the-idb-initiative-too-good-to-waste-call-for-proposals-received-230-proposals-f/1476364899822306</t>
+        </is>
+      </c>
+      <c r="S319" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T319" t="inlineStr">
+        <is>
+          <t>Iniciativa del IDB 'Too Good to Waste' que convoca a propuestas sobre economía circular, enfocada en reutilización, reprocesamiento y reintegración de materiales a ciclos productivos. Según fuente, recibió 230 propuestas.</t>
+        </is>
+      </c>
+      <c r="U319" t="inlineStr">
+        <is>
+          <t>Altamente relevante: el nombre y descripción alinean directamente con los pilares de Visión Circular (cierre de ciclo, reutilización, cadenas circulares, ecodiseño).</t>
+        </is>
+      </c>
+      <c r="V319" t="inlineStr">
+        <is>
+          <t>Pilotos empresariales de reutilización; Ecodiseño para reciclabilidad; Modelos de negocio basados en ciclo cerrado; Inclusión de actores en cadenas reversas; REP operativo</t>
+        </is>
+      </c>
+      <c r="W319" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="X319" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y319" t="inlineStr">
+        <is>
+          <t>Empresas ANDI; Gremios de manufactura; Recicladores y cooperativas; Universidades; Centros tecnológicos</t>
+        </is>
+      </c>
+      <c r="Z319" t="inlineStr">
+        <is>
+          <t>La convocatoria ya recibió 230 propuestas (según post de Facebook de 2017-2018 aproximadamente); es probable que ya esté cerrada o haya evolucionado a otra fase. Requiere verificación urgente.</t>
+        </is>
+      </c>
+      <c r="AA319" t="inlineStr">
+        <is>
+          <t>Verificar si 'Too Good to Waste' sigue abierta o si IDB ha lanzado iteración actualizada; buscar en página oficial del IDB versión actual</t>
+        </is>
+      </c>
+      <c r="AB319" t="inlineStr">
+        <is>
+          <t>Acceder a https://www.iadb.org y buscar 'Too Good to Waste' o convocatorias circulares activas; contactar IDB directamente</t>
+        </is>
+      </c>
+      <c r="AC319" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos; Inteligencia de negocios</t>
+        </is>
+      </c>
+      <c r="AD319" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE319" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF319" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG319" t="inlineStr">
+        <is>
+          <t>El post de Facebook sugiere que la convocatoria ya cerró (dice 'received' 230 proposals). Incluida porque el nombre y tema son altamente relevantes, pero requiere urgente verificación de vigencia. Podría haber sido reemplazada por otro programa del IDB. | Fuente fuera del listado oficial conocido (facebook.com): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH319" t="inlineStr">
+        <is>
+          <t>b3f66b336e8dd90d</t>
+        </is>
+      </c>
+      <c r="AI319" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>VC-0319</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF) - Readiness Support for Colombia</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Green Climate Fund (GCF)</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Fondo climático</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Internacional (sede en Corea del Sur)</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>Países en desarrollo, incluyendo Colombia</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Clima y finanzas climáticas</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>Movilización de finanzas climáticas, AFOLU (Agricultura, Silvicultura y Otros Usos del Suelo), preparación institucional</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>Financiamiento climático; Asistencia técnica; Cooperación técnica</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>7.1 millones USD aprobados para Colombia (histórico); montos específicos por convocatoria no especificados</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>Típicamente sí, según línea de proyecto</t>
+        </is>
+      </c>
+      <c r="N320" t="inlineStr">
+        <is>
+          <t>Abierta permanentemente (convocatorias por línea)</t>
+        </is>
+      </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>No especificado (depende de convocatoria específica)</t>
+        </is>
+      </c>
+      <c r="P320" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q320" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R320" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/countries/colombia</t>
+        </is>
+      </c>
+      <c r="S320" t="inlineStr">
+        <is>
+          <t>https://www.greenclimate.fund/document/advance-mobilization-climate-finance-colombia-s-afolu-sector-through-direct-access-entity; https://www.greenclimate.fund/document/readiness-agreement-colombia-col-rs-001</t>
+        </is>
+      </c>
+      <c r="T320" t="inlineStr">
+        <is>
+          <t>El Green Climate Fund ofrece financiamiento climático a través de Readiness Grants y proyectos directos para países en desarrollo como Colombia. Actualmente ha desembolsado $568.97M de $740.71M aprobados globalmente. Colombia cuenta con $7.1M aprobados en apoyo de preparación y 15 proyectos activos.</t>
+        </is>
+      </c>
+      <c r="U320" t="inlineStr">
+        <is>
+          <t>Altamente relevante para financiar proyectos de economía circular vinculados a reducción de emisiones, reciclaje de plásticos, ecodiseño y transición a modelos circulares en sectores como envases y empaques, especialmente si se articulan con AFOLU o cadenas de valor sostenibles.</t>
+        </is>
+      </c>
+      <c r="V320" t="inlineStr">
+        <is>
+          <t>Financiamiento de pilotos empresariales en reciclaje y economía circular; Preparación de políticas de economía circular y REP; Fortalecimiento de modelos de negocio circulares con inclusión de recicladores; Proyectos de ecodiseño en envases/empaques con co-beneficios climáticos.</t>
+        </is>
+      </c>
+      <c r="W320" t="inlineStr">
+        <is>
+          <t>Ser entidad acreditada ante GCF (agencias ejecutoras nacionales o internacionales); Alineación con NDC de Colombia; Reducción de emisiones o resiliencia climática demostrable; Alineación con prioridades nacionales de cambio climático.</t>
+        </is>
+      </c>
+      <c r="X320" t="inlineStr">
+        <is>
+          <t>Propuesta de proyecto con análisis de impacto climático; Plan de implementación; Marco de seguimiento; Evaluación de riesgos ambientales y sociales; Presupuesto detallado; Cartas de co-financiamiento.</t>
+        </is>
+      </c>
+      <c r="Y320" t="inlineStr">
+        <is>
+          <t>UNDP Colombia (socio clave); Ministerio de Ambiente y Desarrollo Sostenible (MADS); Entidades acreditadas nacionales; Gremios como ANDI; Universidades y centros tecnológicos; Cooperativas de recicladores.</t>
+        </is>
+      </c>
+      <c r="Z320" t="inlineStr">
+        <is>
+          <t>Proceso de acreditación puede ser lento; Requiere co-financiamiento significativo; Competencia alta a nivel global; Ciclos de aprobación extensos.</t>
+        </is>
+      </c>
+      <c r="AA320" t="inlineStr">
+        <is>
+          <t>Identificar líneas de proyecto de Visión Circular con potencial de reducción de emisiones; Contactar a agencias acreditadas ante GCF para evaluar acceso; Preparar mapeo de alineación con NDC de Colombia; Iniciar diálogos con UNDP y MADS para identificar oportunidades de co-financiamiento.</t>
+        </is>
+      </c>
+      <c r="AB320" t="inlineStr">
+        <is>
+          <t>1. Revisar convocatorias activas en https://www.greenclimate.fund/; 2. Contactar agencia ejecutora acreditada en Colombia; 3. Preparar brief de elegibilidad de proyecto Visión Circular; 4. Verificar fechas de cierre de líneas abiertas actualmente.</t>
+        </is>
+      </c>
+      <c r="AC320" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos / Alianzas Estratégicas; Especialista en Financiamiento Climático</t>
+        </is>
+      </c>
+      <c r="AD320" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE320" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF320" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG320" t="inlineStr">
+        <is>
+          <t>GCF es fuente de financiamiento de alto potencial para Visión Circular. Los documentos indican readiness agreements activos con Colombia (COL-RS-001) y programas como Amazonia Viva ya en ejecución. Se infiere que hay ventanas abiertas aunque fechas específicas no aparecen en búsqueda. Requiere verificar convocatorias activas hoy.</t>
+        </is>
+      </c>
+      <c r="AH320" t="inlineStr">
+        <is>
+          <t>209fe5922bf88df9</t>
+        </is>
+      </c>
+      <c r="AI320" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>VC-0320</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>GEF Small Grants Program CSO Challenge Program</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Global Environment Facility (GEF), liderado por International Union for Conservation of Nature (IUCN)</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Fondo ambiental</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Global (182 países miembros)</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Colombia y América Latina (GEF es fondo global con operaciones en región)</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Sostenibilidad ambiental, cambio climático, biodiversidad</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>Economía circular, gestión de residuos, soluciones ambientales innovadoras lideradas por sociedad civil</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cooperación técnica; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>Hasta USD 300,000 por proyecto; Fondo total USD 10 millones</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N321" t="inlineStr">
+        <is>
+          <t>Junio 2026 (lanzamiento oficial confirmado)</t>
+        </is>
+      </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P321" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q321" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R321" t="inlineStr">
+        <is>
+          <t>https://www.thegef.org/what-we-do/topics/gef-small-grants-program</t>
+        </is>
+      </c>
+      <c r="S321" t="inlineStr">
+        <is>
+          <t>https://iucn.org/press-release/202510/new-gef-programme-set-deliver-grants-usd-300000-civil-society-led</t>
+        </is>
+      </c>
+      <c r="T321" t="inlineStr">
+        <is>
+          <t>El GEF SGP Challenge Program es una iniciativa de USD 10 millones que financia hasta USD 300,000 por proyecto para organizaciones de sociedad civil que desarrollen soluciones ambientales innovadoras y escalables. Abierto a CSOs locales en países GEF, incluyendo Colombia, con énfasis en transformación ambiental inclusiva y liderada por comunidades.</t>
+        </is>
+      </c>
+      <c r="U321" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: el programa financia soluciones ambientales innovadoras que pueden incluir economía circular, gestión de residuos, reciclaje y modelos de negocio sostenibles. Alineado con objetivos de Visión Circular en inclusión de actores locales y escalamiento de pilotos.</t>
+        </is>
+      </c>
+      <c r="V321" t="inlineStr">
+        <is>
+          <t>Pilotos de economía circular territorial; Modelos de negocio circulares liderados por recicladores formalizados; Ecodiseño y reciclabilidad de envases/empaques; Gestión integral de residuos en territorios; Inclusión de recicladores en cadenas de valor circular.</t>
+        </is>
+      </c>
+      <c r="W321" t="inlineStr">
+        <is>
+          <t>Ser organización de sociedad civil registrada (CSO); estar operando en país elegible (Colombia aplica); propuesta debe demostrar innovación, escalabilidad y impacto ambiental comprobable; alineación con prioridades GEF (biodiversidad, clima, aguas, degradación de tierras, químicos).</t>
+        </is>
+      </c>
+      <c r="X321" t="inlineStr">
+        <is>
+          <t>No especificado (típicamente: propuesta técnica, presupuesto detallado, evidencia legal de CSO, carta de apoyo de autoridades locales, plan de sostenibilidad)</t>
+        </is>
+      </c>
+      <c r="Y321" t="inlineStr">
+        <is>
+          <t>ANDI como coordinador de alianzas empresariales; Universidades y centros tecnológicos colombianos; Autoridades ambientales territoriales (CORPAS, municipios); Gremios de recicladores; Organizaciones ambientales locales; UNDP como socio implementador en región.</t>
+        </is>
+      </c>
+      <c r="Z321" t="inlineStr">
+        <is>
+          <t>Fecha de lanzamiento es junio 2026 (futura); detalles específicos de aplicación aún no disponibles; competencia alta esperada por fondos limitados; requisitos finales de elegibilidad pendientes de publicación.</t>
+        </is>
+      </c>
+      <c r="AA321" t="inlineStr">
+        <is>
+          <t>Asegurar que ANDI y aliados locales se registren en plataforma GEF cuando abra; preparar cartera de proyectos de Visión Circular que demuestren innovación, escalabilidad e impacto; establecer alianzas con CSOs locales fuertes que puedan liderar aplicación; monitorear publicaciones GEF/IUCN para detalles de convocatoria.</t>
+        </is>
+      </c>
+      <c r="AB321" t="inlineStr">
+        <is>
+          <t>1) Verificar elegibilidad de ANDI y CSO aliados en plataforma GEF (www.thegef.org); 2) Contactar oficina regional GEF/UNDP para Colombia; 3) Preparar resumen ejecutivo de 2-3 proyectos Visión Circular candidatos (modelo circular territorial, inclusión de recicladores, ecodiseño); 4) Registrar en alertas GEF para convocatoria formal 2026.</t>
+        </is>
+      </c>
+      <c r="AC321" t="inlineStr">
+        <is>
+          <t>Coordinación de proyectos e innovación; Alianzas estratégicas con instituciones internacionales</t>
+        </is>
+      </c>
+      <c r="AD321" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE321" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF321" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG321" t="inlineStr">
+        <is>
+          <t>Fuente oficial de GEF y comunicado de prensa IUCN confirman programa activo. Inferencia: economía circular y gestión de residuos son temas GEF priorizados. La fecha de lanzamiento (junio 2026) es futura pero el programa ya tiene asignación de fondos. Requiere seguimiento cercano para detalles de elegibilidad específica de Colombia y tipos de proyecto.</t>
+        </is>
+      </c>
+      <c r="AH321" t="inlineStr">
+        <is>
+          <t>ed5fef1e034d96d9</t>
+        </is>
+      </c>
+      <c r="AI321" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>VC-0321</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>EUROCLIMA+ Eje Economía Circular Regional</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Comisión Europea (Unión Europea), a través de programa EUROCLIMA+</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Cooperación bilateral / Multilateral</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (incluyendo Colombia)</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Economía circular, transición verde, sostenibilidad</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>Gestión de residuos y aguas residuales; Eficiencia en uso de recursos; Modelos de negocio sostenibles; Coordinación regional para transición ambiental</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>Cooperación técnica; Cooperación multilateral; Asistencia técnica; Fortalecimiento institucional</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N322" t="inlineStr">
+        <is>
+          <t>Abierta (programa en vigencia)</t>
+        </is>
+      </c>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P322" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q322" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R322" t="inlineStr">
+        <is>
+          <t>https://www.fiap.gob.es/noticias/euroclima-impulsa-la-coordinacion-regional-para-avanzar-en-la-transicion-verde-en-america-latina-y-el-caribe</t>
+        </is>
+      </c>
+      <c r="S322" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="T322" t="inlineStr">
+        <is>
+          <t>EUROCLIMA+ es programa de cooperación de la Unión Europea que impulsa coordinación regional en América Latina y el Caribe para transición verde. Posiciona economía circular como eje central, con énfasis en gestión de residuos, eficiencia de recursos y modelos de negocio sostenibles.</t>
+        </is>
+      </c>
+      <c r="U322" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: programa explícitamente prioriza economía circular, gestión de residuos, eficiencia de recursos y modelos de negocio sostenibles en América Latina. Alineación directa con temas de Visión Circular ANDI.</t>
+        </is>
+      </c>
+      <c r="V322" t="inlineStr">
+        <is>
+          <t>Coordinación regional de políticas de economía circular; Sistemas territoriales de gestión de residuos y reciclaje; Modelos de negocio circular para PyMEs y gremios; Eficiencia de recursos en cadenas de valor de envases/empaques; Asistencia técnica a gobiernos locales en transición circular.</t>
+        </is>
+      </c>
+      <c r="W322" t="inlineStr">
+        <is>
+          <t>Entidades públicas de América Latina (gobiernos, ministerios); potencial acceso para gremios, universidades y actores privados vía alianzas con gobiernos; propuestas con enfoque regional y coordinación multinacional priorizadas.</t>
+        </is>
+      </c>
+      <c r="X322" t="inlineStr">
+        <is>
+          <t>No especificado (típicamente: propuesta técnica con socio gubernamental, análisis de contexto regional, plan de trabajo, presupuesto, equipo especializado)</t>
+        </is>
+      </c>
+      <c r="Y322" t="inlineStr">
+        <is>
+          <t>Ministerios de Ambiente/Sostenibilidad de Colombia; Gobiernos locales; ANDI como coordinador de sector privado; Gremios de reciclaje y gestión de residuos; Universidades con investigación en economía circular; Agencias ambientales regionales.</t>
+        </is>
+      </c>
+      <c r="Z322" t="inlineStr">
+        <is>
+          <t>URL proporcionada es comunicado de noticias sin detalles de convocatoria abierta; no se especifica si hay llamado activo ni montos disponibles; se requiere verificar cómo acceden gremios/sector privado (posiblemente solo vía gobiernos); marco temporal no está claramente definido.</t>
+        </is>
+      </c>
+      <c r="AA322" t="inlineStr">
+        <is>
+          <t>Contactar directamente a coordinación EUROCLIMA+ en región (probablemente a través de oficina en Colombia o punto focal UE); explorar alianza con Ministerio de Ambiente o autoridades locales para posicionar proyectos Visión Circular; solicitar información sobre mecanismos de acceso para gremios empresariales.</t>
+        </is>
+      </c>
+      <c r="AB322" t="inlineStr">
+        <is>
+          <t>1) Identificar punto focal EUROCLIMA+ para Colombia (búsqueda en www.euroclima.org o sitios UE); 2) Contactar embajada/delegación UE en Colombia; 3) Indagar sobre convocatorias abiertas específicas en economía circular; 4) Preparar propuesta piloto de Visión Circular con socio gubernamental.</t>
+        </is>
+      </c>
+      <c r="AC322" t="inlineStr">
+        <is>
+          <t>Alianzas estratégicas internacionales; Coordinación con gobiernos y autoridades ambientales</t>
+        </is>
+      </c>
+      <c r="AD322" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE322" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF322" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG322" t="inlineStr">
+        <is>
+          <t>Información proviene de comunicado oficial de FIAP (Federación Iberoamericana de Asociaciones de Parques y Áreas Protegidas, colaboradora UE). Economía circular es eje confirmado de EUROCLIMA+. Inferencia: programa está en vigencia pero fuente no especifica convocatorias abiertas ni mecanismos de acceso para sector privado/gremios. Requiere verificación de elegibilidad directa y convocatorias activas. | Fuente fuera del listado oficial conocido (fiap.gob.es): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH322" t="inlineStr">
+        <is>
+          <t>6f88e1c2b00a6d34</t>
+        </is>
+      </c>
+      <c r="AI322" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>VC-0322</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Programa Euroclima - Convocatoria de Subvenciones para Proyectos de Economía Circular</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Unión Europea (UE) a través de Euroclima, implementado por Expertise France e INTPA</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Cooperación multilateral</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>América Latina y el Caribe (Programa Euroclima cubre región; confirmación para Colombia pendiente)</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Economía circular</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>Diseño e implementación de proyectos de economía circular; diálogo interinstitucional; posicionamiento político de sostenibilidad</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>Grant no reembolsable; Cooperación técnica; Asistencia técnica</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="N323" t="inlineStr">
+        <is>
+          <t>No especificado (inferido como vigente según publicación en redes 2025)</t>
+        </is>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="P323" t="inlineStr">
+        <is>
+          <t>Requiere verificación manual</t>
+        </is>
+      </c>
+      <c r="Q323" t="inlineStr">
+        <is>
+          <t>Requiere verificación</t>
+        </is>
+      </c>
+      <c r="R323" t="inlineStr">
+        <is>
+          <t>https://expertise-france.gestmax.fr/_expertise_france/public_files/tdr-experto-a-guatemala-economia-circular.pdf</t>
+        </is>
+      </c>
+      <c r="S323" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DPHIjaLjjUq</t>
+        </is>
+      </c>
+      <c r="T323" t="inlineStr">
+        <is>
+          <t>Euroclima (financiado por la UE) financia el diseño e implementación de proyectos de economía circular en América Latina mediante un enfoque de diálogo país orientado al diálogo interinstitucional y político. La convocatoria está abierta y busca promover prácticas circulares posicionando la sostenibilidad como eje estratégico.</t>
+        </is>
+      </c>
+      <c r="U323" t="inlineStr">
+        <is>
+          <t>Altamente pertinente: se alinea directamente con los objetivos de Visión Circular (economía circular, diálogo con autoridades, empresas y gremios) y financia proyectos diseñados bajo metodología de diálogo país.</t>
+        </is>
+      </c>
+      <c r="V323" t="inlineStr">
+        <is>
+          <t>Modelos de negocio circulares; Pilotos empresariales en economía circular; Articulación multi-actor (empresas, gremios, universidades, autoridades); Reformas políticas para economía circular; Inclusión de actores en cadenas circulares</t>
+        </is>
+      </c>
+      <c r="W323" t="inlineStr">
+        <is>
+          <t>No especificado (requiere verificación en portal oficial de Euroclima)</t>
+        </is>
+      </c>
+      <c r="X323" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="Y323" t="inlineStr">
+        <is>
+          <t>ANDI, gremios colombianos, universidades, centros tecnológicos, autoridades ambientales, cooperativas de recicladores, empresas de envases y empaques</t>
+        </is>
+      </c>
+      <c r="Z323" t="inlineStr">
+        <is>
+          <t>Información fragmentaria: no hay URL oficial completa de la convocatoria, fechas de cierre no especificadas, elegibilidad exacta para Colombia no confirmada explícitamente</t>
+        </is>
+      </c>
+      <c r="AA323" t="inlineStr">
+        <is>
+          <t>Contactar inmediatamente a Euroclima y Expertise France para solicitar términos de referencia completos, cronograma exacto y elegibilidad de Colombia. Preparar concepto de proyecto alineado con diálogo país.</t>
+        </is>
+      </c>
+      <c r="AB323" t="inlineStr">
+        <is>
+          <t>1) Acceder a portal oficial de Euroclima (https://www.euroclima.info o similar) para confirmar convocatoria vigente; 2) Contactar focal point en Colombia de Euroclima/UE; 3) Validar si ANDI puede aplicar directamente o requiere alianza con entidad local</t>
+        </is>
+      </c>
+      <c r="AC323" t="inlineStr">
+        <is>
+          <t>Coordinación de Proyectos y Alianzas; Responsable de Cooperación Internacional</t>
+        </is>
+      </c>
+      <c r="AD323" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE323" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF323" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AG323" t="inlineStr">
+        <is>
+          <t>Fuente: Post de Instagram de Euroclima (fecha ~enero 2025) y documento de TDR para experto en Guatemala sugieren programa activo. Sin embargo, no hay URL oficial completa de convocatoria ni términos explícitos. La metodología de 'diálogo país' es característica de Euroclima. Requiere verificación urgente de portal oficial. | Fuente fuera del listado oficial conocido (expertise-france.gestmax.fr): verificar oficialidad</t>
+        </is>
+      </c>
+      <c r="AH323" t="inlineStr">
+        <is>
+          <t>5078fe6a3b740dd4</t>
+        </is>
+      </c>
+      <c r="AI323" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>

</xml_diff>